<commit_message>
Highlight fixed page bookmarks with custom star icon
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF137561-8444-408F-878E-7F0F58BEB7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B13DAD-DCE5-4F54-9708-BE17600E339D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11529" yWindow="19650" windowWidth="21901" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9260" yWindow="19686" windowWidth="24170" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
   <si>
     <t>0</t>
     <phoneticPr fontId="4"/>
@@ -390,6 +390,45 @@
     <rPh sb="23" eb="24">
       <t>カ</t>
     </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>★印を固定ページブックマークの印として使えないか？</t>
+    <rPh sb="1" eb="2">
+      <t>ジルシ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>コテイ</t>
+    </rPh>
+    <rPh sb="15" eb="16">
+      <t>シルシ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>ツカ</t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>H</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>5fdf7a0aa</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>Git Commit</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>BookControl.cs
+BookControlProxy.cs
+IBookControl.cs
+BookmarkCollectionService.cs
+CreateBookmarkCommand.cs
+ToggleBookmarkCommand.cs
+FolderListBox.xaml.cs
+BookAccessor.cs</t>
     <phoneticPr fontId="4"/>
   </si>
 </sst>
@@ -472,7 +511,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -513,6 +552,12 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -799,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
     <col min="1" max="1" width="4.23046875" style="2" customWidth="1"/>
@@ -807,15 +852,19 @@
     <col min="4" max="4" width="68.921875" style="3" customWidth="1"/>
     <col min="5" max="5" width="4.4609375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="59.765625" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="9.23046875" style="1"/>
+    <col min="7" max="7" width="9.921875" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="C1" s="14" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="33.75">
+      <c r="G1" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="33.75">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -829,7 +878,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="B3" s="6" t="s">
         <v>29</v>
       </c>
@@ -837,7 +886,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7">
       <c r="B4" s="6" t="s">
         <v>30</v>
       </c>
@@ -845,7 +894,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="B5" s="6" t="s">
         <v>31</v>
       </c>
@@ -853,7 +902,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
@@ -861,7 +910,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="B7" s="6" t="s">
         <v>33</v>
       </c>
@@ -869,7 +918,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="B8" s="6" t="s">
         <v>34</v>
       </c>
@@ -877,7 +926,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="B9" s="6" t="s">
         <v>35</v>
       </c>
@@ -885,7 +934,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="B10" s="6" t="s">
         <v>36</v>
       </c>
@@ -893,7 +942,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11" s="2" t="s">
         <v>1</v>
       </c>
@@ -901,7 +950,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="33.75">
+    <row r="12" spans="1:7" ht="33.75">
       <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
@@ -915,7 +964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="33.75">
+    <row r="13" spans="1:7" ht="33.75">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
@@ -932,7 +981,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="67.45">
+    <row r="14" spans="1:7" ht="67.45">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
@@ -949,7 +998,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="50.6">
+    <row r="15" spans="1:7" ht="50.6">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
@@ -963,7 +1012,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="84.3">
+    <row r="16" spans="1:7" ht="67.45">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
@@ -980,7 +1029,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:7">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
@@ -997,7 +1046,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:7">
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
@@ -1011,7 +1060,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:7">
       <c r="A19" s="2" t="s">
         <v>8</v>
       </c>
@@ -1025,7 +1074,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="50.6">
+    <row r="20" spans="1:7" ht="33.75">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1039,7 +1088,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="50.6">
+    <row r="21" spans="1:7" ht="50.6">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
@@ -1056,7 +1105,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="50.6">
+    <row r="22" spans="1:7" ht="33.75">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
@@ -1070,7 +1119,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="33.75">
+    <row r="23" spans="1:7" ht="134.9">
       <c r="A23" s="13" t="s">
         <v>40</v>
       </c>
@@ -1083,8 +1132,14 @@
       <c r="E23" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="33.75">
+      <c r="F23" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="33.75">
       <c r="A24" s="13" t="s">
         <v>44</v>
       </c>
@@ -1095,7 +1150,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:7">
       <c r="A25" s="13" t="s">
         <v>47</v>
       </c>
@@ -1103,12 +1158,23 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:7">
       <c r="A26" s="13" t="s">
         <v>48</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enable Ctrl+D bookmark making for multiple bookshelf selections
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B13DAD-DCE5-4F54-9708-BE17600E339D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9115AFA1-8FFA-467D-9F5B-07C5F3A8131F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9260" yWindow="19686" windowWidth="24170" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
   <si>
     <t>0</t>
     <phoneticPr fontId="4"/>
@@ -116,13 +116,6 @@
     </rPh>
     <rPh sb="55" eb="57">
       <t>ドウキ</t>
-    </rPh>
-    <phoneticPr fontId="4"/>
-  </si>
-  <si>
-    <t>未</t>
-    <rPh sb="0" eb="1">
-      <t>ミ</t>
     </rPh>
     <phoneticPr fontId="4"/>
   </si>
@@ -429,6 +422,41 @@
 ToggleBookmarkCommand.cs
 FolderListBox.xaml.cs
 BookAccessor.cs</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>7640e4cc9</t>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>次回の課題</t>
+    <rPh sb="0" eb="2">
+      <t>ジカイ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>カダイ</t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>★のアイコンをクリックしたときの動作を追加する。</t>
+    <rPh sb="16" eb="18">
+      <t>ドウサ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>ツイカ</t>
+    </rPh>
+    <phoneticPr fontId="4"/>
+  </si>
+  <si>
+    <t>$ git show --pretty="" --name-only HEAD | xargs -n1 basename
+BookmarkCollectionService.cs
+DarkTheme.json
+MainWindowResourceDictionary.xaml
+FolderItem.cs
+FolderListIcon.cs
+Colors.xaml
+NeeViewProjects.xlsx</t>
     <phoneticPr fontId="4"/>
   </si>
 </sst>
@@ -511,7 +539,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -557,6 +585,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -844,192 +878,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
     <col min="1" max="1" width="4.23046875" style="2" customWidth="1"/>
     <col min="2" max="3" width="4.69140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="68.921875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="59.69140625" style="3" customWidth="1"/>
     <col min="5" max="5" width="4.4609375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="59.765625" style="5" customWidth="1"/>
     <col min="7" max="7" width="9.921875" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.23046875" style="1"/>
+    <col min="8" max="8" width="9.23046875" style="18" customWidth="1"/>
+    <col min="9" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="C1" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="33.75">
+        <v>53</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="33.75">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="B3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="B4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="B5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="B6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="B7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="B8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="B9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="B10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="B10" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="C10" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="33.75">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="33.75">
       <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="33.75">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="33.75">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="67.45">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="67.45">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="50.6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="50.6">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="67.45">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="67.45">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>20</v>
-      </c>
       <c r="F16" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
@@ -1037,144 +1072,149 @@
         <v>15</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="33.75">
+      <c r="E19" s="12"/>
+    </row>
+    <row r="20" spans="1:8" ht="33.75">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="50.6">
+      <c r="E20" s="11"/>
+    </row>
+    <row r="21" spans="1:8" ht="50.6">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="33.75">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="33.75">
       <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="134.9">
+      <c r="A23" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="33.75">
+      <c r="A24" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="C24" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="33.75">
+      <c r="A26" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="134.9">
+      <c r="A27" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" ht="134.9">
-      <c r="A23" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="9" t="s">
+      <c r="F27" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="G23" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="33.75">
-      <c r="A24" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>51</v>
+      <c r="H27" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Fix] Bookshelf thumbnail refresh after SetThumbnail
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9115AFA1-8FFA-467D-9F5B-07C5F3A8131F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{A363630C-97EC-4BA7-B6C6-9AC32AC6B2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9260" yWindow="19686" windowWidth="24170" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,82 +26,82 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
   <si>
     <t>0</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>9</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>B</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>ルート検索(トグル)の機能追加</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>検索窓にキーワードを打ち込んだら、currentフォルダーから下を対象に検索を開始するのやけど、ルート検索にしたら、ルートに設定してあるフォルダー(「本棚」なら、ホーム・ディレクトリあたりが適任。「ブックマーク」なら、ルート)からの検索になる仕様追加変更の検討。</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>NeeView内削除 → 関連ブクマ削除</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>00</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>01</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>ブックマーク・リングの再設定追加機能</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>メインビュー → ブックマークフォルダー D&amp;D登録</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>「本棚」パネルのタイトルバーにブックタイトルを表示。
@@ -117,14 +118,14 @@
     <rPh sb="55" eb="57">
       <t>ドウキ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>完了</t>
     <rPh sb="0" eb="2">
       <t>カンリョウ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>サムネ・アイコン表示モードでの長すぎるファイル名の最後尾からちょい手前を省略する機能</t>
@@ -143,7 +144,7 @@
     <rPh sb="36" eb="38">
       <t>ショウリャク</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>FolderTreeViewで「新しいフォルダー」コンテキストメニューをクリックしたときの挙動改善</t>
@@ -156,7 +157,7 @@
     <rPh sb="47" eb="49">
       <t>カイゼン</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>■ブックマークをブクマ・フォルダーからブクマ・フォルダーへD&amp;Dでポイしたら、ポイした先にブクマは移動。
@@ -182,12 +183,12 @@
     <rPh sb="110" eb="111">
       <t>サキ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>■ TreeView→ListBox同期経路を探索
 ■ListBox表示切替の正式ルート</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>■ブックマークのコピーと貼り付け
@@ -204,7 +205,7 @@
     <rPh sb="38" eb="40">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>「ブックマーク」パネルのに「←→」ボタンを追加。
@@ -224,59 +225,59 @@
     <rPh sb="61" eb="63">
       <t>デキ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>Bookmark.OpenPageMode（Resume / Fixed）をちゃんと動かすために、NeeViewの「本を開く流れ」を逆流調査してた。</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>private void FolderList_KeyDown(object? sender, KeyEventArgs e)</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>いまの設計では「本棚」パネルも「ページ」パネルもサムネ表示したときのサムネサイズはどちらも同じサイズで縛られてる。</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>C</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>Ctrl + Shift + Dで「ブックマーク」パネルでSelectedなフォルダーに固定ページブクマを作成する</t>
@@ -286,19 +287,19 @@
     <rPh sb="53" eb="55">
       <t>サクセイ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>AI</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>〇</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>D</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>パネルをフローティングにしたときに、ショートカットキーで各パネルへフォーカスしてアクティブな状態にしたい。</t>
@@ -308,7 +309,7 @@
     <rPh sb="46" eb="48">
       <t>ジョウタイ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>■「←→」キー打鍵だけでサムネ表示時のフォーカス・ブック移動を最初から最後までシームレスに移動できるようにする
@@ -343,15 +344,15 @@
     <rPh sb="67" eb="68">
       <t>カエ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>F</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>G</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>複数ファイルのCtrl+DとCtrl+Shift+Dの動作が単一ファイルしか操作されてなかった。</t>
@@ -367,7 +368,7 @@
     <rPh sb="38" eb="40">
       <t>ソウサ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>第一ホームと第二ホーム、第三ホームまでアイコン化</t>
@@ -383,7 +384,7 @@
     <rPh sb="23" eb="24">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>★印を固定ページブックマークの印として使えないか？</t>
@@ -399,19 +400,19 @@
     <rPh sb="19" eb="20">
       <t>ツカ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>H</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>5fdf7a0aa</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>Git Commit</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>BookControl.cs
@@ -422,11 +423,11 @@
 ToggleBookmarkCommand.cs
 FolderListBox.xaml.cs
 BookAccessor.cs</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>7640e4cc9</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
   </si>
   <si>
     <t>次回の課題</t>
@@ -436,35 +437,230 @@
     <rPh sb="3" eb="5">
       <t>カダイ</t>
     </rPh>
-    <phoneticPr fontId="4"/>
-  </si>
-  <si>
-    <t>★のアイコンをクリックしたときの動作を追加する。</t>
-    <rPh sb="16" eb="18">
-      <t>ドウサ</t>
-    </rPh>
-    <rPh sb="19" eb="21">
-      <t>ツイカ</t>
-    </rPh>
-    <phoneticPr fontId="4"/>
-  </si>
-  <si>
-    <t>$ git show --pretty="" --name-only HEAD | xargs -n1 basename
-BookmarkCollectionService.cs
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>b4dc93aa4</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>make-links.ps1の運用を開始する</t>
+    <rPh sb="15" eb="17">
+      <t>ウンヨウ</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>カイシ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>BookmarkCollectionService.cs
 DarkTheme.json
 MainWindowResourceDictionary.xaml
 FolderItem.cs
 FolderListIcon.cs
 Colors.xaml
 NeeViewProjects.xlsx</t>
-    <phoneticPr fontId="4"/>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>CreateBookmarkCommand.cs
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t xml:space="preserve">★のアイコンをクリックしたときの動作を追加する。
+</t>
+    <rPh sb="16" eb="18">
+      <t>ドウサ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>ツイカ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>その他</t>
+    <rPh sb="2" eb="3">
+      <t>タ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>■本家からの返事。
+ShiftとかCtrlとかを同時押しのばあいの「←→」をどうするか？</t>
+    <rPh sb="1" eb="3">
+      <t>ホンケ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ヘンジ</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>ドウジ</t>
+    </rPh>
+    <rPh sb="26" eb="27">
+      <t>オ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>J</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？</t>
+    <rPh sb="9" eb="10">
+      <t>カズ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>ホンダナ</t>
+    </rPh>
+    <rPh sb="20" eb="21">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t>ミギカタ</t>
+    </rPh>
+    <rPh sb="25" eb="27">
+      <t>ヒョウジ</t>
+    </rPh>
+    <rPh sb="31" eb="32">
+      <t>イロ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>https://chatgpt.com/c/6a2f9616-be38-83e8-b9d9-edc6d1622263#12-1</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>K</t>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>「本棚」でサムネの画像を指定するコンテキストメニューを実行したところ、不具合発生。
+「現在のページをサムネイルに設定する」メニュー項目がクリックしても本のサムネ用画像の指定変更がサムネに反映されない。</t>
+    <rPh sb="1" eb="3">
+      <t>ホンダナ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ガゾウ</t>
+    </rPh>
+    <rPh sb="12" eb="14">
+      <t>シテイ</t>
+    </rPh>
+    <rPh sb="27" eb="29">
+      <t>ジッコウ</t>
+    </rPh>
+    <rPh sb="35" eb="38">
+      <t>フグアイ</t>
+    </rPh>
+    <rPh sb="38" eb="40">
+      <t>ハッセイ</t>
+    </rPh>
+    <rPh sb="43" eb="45">
+      <t>ゲンザイ</t>
+    </rPh>
+    <rPh sb="56" eb="58">
+      <t>セッテイ</t>
+    </rPh>
+    <rPh sb="65" eb="67">
+      <t>コウモク</t>
+    </rPh>
+    <rPh sb="75" eb="76">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="80" eb="81">
+      <t>ヨウ</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>ガゾウ</t>
+    </rPh>
+    <rPh sb="84" eb="86">
+      <t>シテイ</t>
+    </rPh>
+    <rPh sb="86" eb="88">
+      <t>ヘンコウ</t>
+    </rPh>
+    <rPh sb="93" eb="95">
+      <t>ハンエイホンダナヒョウジヒョウジドウキ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>行の一番端、右端でも左端でも、そこでShiftを押しながら、←→キーを叩いたら、次の行(下の段)、または前の行(上の段)に選択状態を維持したままカーソルが動いた。</t>
+    <rPh sb="0" eb="1">
+      <t>ギョウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>イチバン</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ハシ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ミギハジ</t>
+    </rPh>
+    <rPh sb="10" eb="12">
+      <t>ヒダリハジ</t>
+    </rPh>
+    <rPh sb="24" eb="25">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="35" eb="36">
+      <t>タタ</t>
+    </rPh>
+    <rPh sb="40" eb="41">
+      <t>ツギ</t>
+    </rPh>
+    <rPh sb="42" eb="43">
+      <t>ギョウ</t>
+    </rPh>
+    <rPh sb="44" eb="45">
+      <t>シタ</t>
+    </rPh>
+    <rPh sb="46" eb="47">
+      <t>ダン</t>
+    </rPh>
+    <rPh sb="52" eb="53">
+      <t>マエ</t>
+    </rPh>
+    <rPh sb="54" eb="55">
+      <t>ギョウ</t>
+    </rPh>
+    <rPh sb="56" eb="57">
+      <t>ウエ</t>
+    </rPh>
+    <rPh sb="58" eb="59">
+      <t>ダン</t>
+    </rPh>
+    <rPh sb="61" eb="63">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="63" eb="65">
+      <t>ジョウタイ</t>
+    </rPh>
+    <rPh sb="66" eb="68">
+      <t>イジ</t>
+    </rPh>
+    <rPh sb="77" eb="78">
+      <t>ウゴ</t>
+    </rPh>
+    <phoneticPr fontId="7"/>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="7"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -494,14 +690,43 @@
       <charset val="128"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
       <sz val="6"/>
       <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -520,12 +745,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -536,65 +755,106 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -878,121 +1138,129 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="1" width="4.23046875" style="2" customWidth="1"/>
-    <col min="2" max="3" width="4.69140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="59.69140625" style="3" customWidth="1"/>
+    <col min="1" max="2" width="3.921875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="51.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="4.4609375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="59.765625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="9.921875" style="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.23046875" style="18" customWidth="1"/>
-    <col min="9" max="16384" width="9.23046875" style="1"/>
+    <col min="6" max="6" width="43.3046875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="9.921875" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="42.15234375" style="15" customWidth="1"/>
+    <col min="9" max="9" width="9.23046875" style="5"/>
+    <col min="10" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
-      <c r="C1" s="14" t="s">
+    <row r="1" spans="1:9">
+      <c r="A1" s="20"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="D1" s="22"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="23" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="33.75">
+      <c r="I1" s="24" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="50.6">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="12" t="s">
         <v>42</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:9">
       <c r="B3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+      <c r="C3" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="B4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+      <c r="C4" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="B5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+      <c r="C5" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="B6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+      <c r="C6" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="B7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+      <c r="C7" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="B8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+      <c r="C8" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="B9" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
+      <c r="C9" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="B10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+      <c r="C10" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="33.75">
+      <c r="C11" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="33.75">
       <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -1002,11 +1270,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="33.75">
+    <row r="13" spans="1:9" ht="33.75">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1019,11 +1287,11 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="67.45">
+    <row r="14" spans="1:9" ht="101.2">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -1036,11 +1304,11 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="50.6">
+    <row r="15" spans="1:9" ht="50.6">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -1049,12 +1317,15 @@
       <c r="E15" s="10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="67.45">
+      <c r="H15" s="19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="101.2">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -1064,14 +1335,14 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1081,46 +1352,47 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:9">
       <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:9">
       <c r="A19" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="12"/>
-    </row>
-    <row r="20" spans="1:8" ht="33.75">
+    </row>
+    <row r="20" spans="1:9" ht="67.45">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="11"/>
-    </row>
-    <row r="21" spans="1:8" ht="50.6">
+    </row>
+    <row r="21" spans="1:9" ht="50.6">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="B21" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>42</v>
       </c>
       <c r="D21" s="9" t="s">
@@ -1133,95 +1405,175 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="33.75">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:9" ht="50.6">
+      <c r="B22" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:9" ht="33.75">
+      <c r="A23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="9" t="s">
+      <c r="B23" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="9" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="134.9">
-      <c r="A23" s="13" t="s">
+    <row r="24" spans="1:9" ht="134.9">
+      <c r="A24" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="B24" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E24" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F24" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G23" s="15" t="s">
+      <c r="G24" s="13" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="33.75">
-      <c r="A24" s="13" t="s">
+    <row r="25" spans="1:9" ht="33.75">
+      <c r="A25" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="B25" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="13" t="s">
+    <row r="26" spans="1:9">
+      <c r="A26" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="B26" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="33.75">
-      <c r="A26" s="13" t="s">
+    <row r="27" spans="1:9" ht="33.75">
+      <c r="A27" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="B27" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="134.9">
-      <c r="A27" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>50</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G27" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="I27" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="G27" s="15" t="s">
+    </row>
+    <row r="28" spans="1:9" ht="118.05">
+      <c r="A28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="G28" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="H27" s="17" t="s">
-        <v>57</v>
+      <c r="H28" s="19" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="33.75">
+      <c r="A29" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="30">
+        <v>0.5</v>
+      </c>
+      <c r="I29" s="26" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="67.45">
+      <c r="A30" s="27" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="30">
+        <v>0.03</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4"/>
+  <phoneticPr fontId="7"/>
+  <hyperlinks>
+    <hyperlink ref="I29" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A11 A12:B20 A2 B2:B10" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Feat] Resume bookmark first in bookmark filename sort
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{A363630C-97EC-4BA7-B6C6-9AC32AC6B2FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FF4C9A-A59C-4EDB-80F5-058FEF5AD40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,82 +25,74 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="80">
   <si>
     <t>0</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>9</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>B</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>ルート検索(トグル)の機能追加</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>検索窓にキーワードを打ち込んだら、currentフォルダーから下を対象に検索を開始するのやけど、ルート検索にしたら、ルートに設定してあるフォルダー(「本棚」なら、ホーム・ディレクトリあたりが適任。「ブックマーク」なら、ルート)からの検索になる仕様追加変更の検討。</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>NeeView内削除 → 関連ブクマ削除</t>
-    <phoneticPr fontId="7"/>
-  </si>
-  <si>
-    <t>00</t>
-    <phoneticPr fontId="7"/>
-  </si>
-  <si>
-    <t>01</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>ブックマーク・リングの再設定追加機能</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>メインビュー → ブックマークフォルダー D&amp;D登録</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>「本棚」パネルのタイトルバーにブックタイトルを表示。
@@ -118,14 +109,14 @@
     <rPh sb="55" eb="57">
       <t>ドウキ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>完了</t>
     <rPh sb="0" eb="2">
       <t>カンリョウ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>サムネ・アイコン表示モードでの長すぎるファイル名の最後尾からちょい手前を省略する機能</t>
@@ -144,7 +135,7 @@
     <rPh sb="36" eb="38">
       <t>ショウリャク</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>FolderTreeViewで「新しいフォルダー」コンテキストメニューをクリックしたときの挙動改善</t>
@@ -157,7 +148,7 @@
     <rPh sb="47" eb="49">
       <t>カイゼン</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>■ブックマークをブクマ・フォルダーからブクマ・フォルダーへD&amp;Dでポイしたら、ポイした先にブクマは移動。
@@ -183,12 +174,12 @@
     <rPh sb="110" eb="111">
       <t>サキ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>■ TreeView→ListBox同期経路を探索
 ■ListBox表示切替の正式ルート</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>■ブックマークのコピーと貼り付け
@@ -205,7 +196,7 @@
     <rPh sb="38" eb="40">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>「ブックマーク」パネルのに「←→」ボタンを追加。
@@ -225,59 +216,59 @@
     <rPh sb="61" eb="63">
       <t>デキ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>Bookmark.OpenPageMode（Resume / Fixed）をちゃんと動かすために、NeeViewの「本を開く流れ」を逆流調査してた。</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>private void FolderList_KeyDown(object? sender, KeyEventArgs e)</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>いまの設計では「本棚」パネルも「ページ」パネルもサムネ表示したときのサムネサイズはどちらも同じサイズで縛られてる。</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>C</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>Ctrl + Shift + Dで「ブックマーク」パネルでSelectedなフォルダーに固定ページブクマを作成する</t>
@@ -287,19 +278,19 @@
     <rPh sb="53" eb="55">
       <t>サクセイ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>AI</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>〇</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>D</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>パネルをフローティングにしたときに、ショートカットキーで各パネルへフォーカスしてアクティブな状態にしたい。</t>
@@ -309,7 +300,7 @@
     <rPh sb="46" eb="48">
       <t>ジョウタイ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>■「←→」キー打鍵だけでサムネ表示時のフォーカス・ブック移動を最初から最後までシームレスに移動できるようにする
@@ -344,15 +335,15 @@
     <rPh sb="67" eb="68">
       <t>カエ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>F</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>G</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>複数ファイルのCtrl+DとCtrl+Shift+Dの動作が単一ファイルしか操作されてなかった。</t>
@@ -368,7 +359,7 @@
     <rPh sb="38" eb="40">
       <t>ソウサ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>第一ホームと第二ホーム、第三ホームまでアイコン化</t>
@@ -384,7 +375,7 @@
     <rPh sb="23" eb="24">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>★印を固定ページブックマークの印として使えないか？</t>
@@ -400,19 +391,19 @@
     <rPh sb="19" eb="20">
       <t>ツカ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>H</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>5fdf7a0aa</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>Git Commit</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>BookControl.cs
@@ -423,25 +414,15 @@
 ToggleBookmarkCommand.cs
 FolderListBox.xaml.cs
 BookAccessor.cs</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>7640e4cc9</t>
-    <phoneticPr fontId="7"/>
-  </si>
-  <si>
-    <t>次回の課題</t>
-    <rPh sb="0" eb="2">
-      <t>ジカイ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>カダイ</t>
-    </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>b4dc93aa4</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>make-links.ps1の運用を開始する</t>
@@ -451,7 +432,7 @@
     <rPh sb="18" eb="20">
       <t>カイシ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>BookmarkCollectionService.cs
@@ -461,12 +442,12 @@
 FolderListIcon.cs
 Colors.xaml
 NeeViewProjects.xlsx</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>CreateBookmarkCommand.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t xml:space="preserve">★のアイコンをクリックしたときの動作を追加する。
@@ -477,14 +458,14 @@
     <rPh sb="19" eb="21">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>その他</t>
     <rPh sb="2" eb="3">
       <t>タ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>■本家からの返事。
@@ -501,11 +482,11 @@
     <rPh sb="26" eb="27">
       <t>オ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>J</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？</t>
@@ -530,15 +511,15 @@
     <rPh sb="33" eb="34">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>https://chatgpt.com/c/6a2f9616-be38-83e8-b9d9-edc6d1622263#12-1</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>K</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>「本棚」でサムネの画像を指定するコンテキストメニューを実行したところ、不具合発生。
@@ -588,7 +569,7 @@
     <rPh sb="93" eb="95">
       <t>ハンエイホンダナヒョウジヒョウジドウキ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>行の一番端、右端でも左端でも、そこでShiftを押しながら、←→キーを叩いたら、次の行(下の段)、または前の行(上の段)に選択状態を維持したままカーソルが動いた。</t>
@@ -649,24 +630,158 @@
     <rPh sb="77" eb="78">
       <t>ウゴ</t>
     </rPh>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="7"/>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Cache.dbの存在を知る</t>
+    <rPh sb="9" eb="11">
+      <t>ソンザイ</t>
+    </rPh>
+    <rPh sb="12" eb="13">
+      <t>シ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>7ca3c5ebb</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>FolderListBox.xaml.cs
+ListBoxThumbnailLoader.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>リセット
+ _shiftSelectionAnchorIndex = -1;
+ _shiftSelectionCurrentIndex = -1;
+■マウスで飛ぶ場合。
+■Shift + ← or Shift + →で選択範囲を開始。途中でShift + ↑の操作をしたときの選択範囲が異常</t>
+    <rPh sb="79" eb="80">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="117" eb="119">
+      <t>トチュウ</t>
+    </rPh>
+    <rPh sb="130" eb="132">
+      <t>ソウサ</t>
+    </rPh>
+    <rPh sb="138" eb="140">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="140" eb="142">
+      <t>ハンイ</t>
+    </rPh>
+    <rPh sb="143" eb="145">
+      <t>イジョウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>対象ファイル。関数。</t>
+    <rPh sb="0" eb="2">
+      <t>タイショウ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>カンスウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>取り組み内容</t>
+    <rPh sb="0" eb="1">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ク</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ナイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>次回の課題</t>
+    <rPh sb="0" eb="2">
+      <t>ジカイ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>カダイ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>https://chatgpt.com/c/6a2fc982-dc44-83ee-8d8d-af34bf9343d3#64</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>L</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>ファイルのファイル名によるソート順についての改善。
+Tmep.zip、Temp(1).zip、Temp(2).zip、Temp(3).zip、Temp(4).zip、…とあると、ソートされた表示は、Temp(1).zip、Temp(2).zip、Temp(3).zip、Temp(4).zip、…、Temp.zipになってしまうこと。これは良くない。
+Tmep.zip、Temp(1).zip、Temp(2).zip、Temp(3).zip、Temp(4).zip、…とこのような順番で表示して欲しい。</t>
+    <rPh sb="9" eb="10">
+      <t>メイ</t>
+    </rPh>
+    <rPh sb="16" eb="17">
+      <t>ジュン</t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t>カイゼン</t>
+    </rPh>
+    <rPh sb="95" eb="97">
+      <t>ヒョウジ</t>
+    </rPh>
+    <rPh sb="170" eb="171">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="240" eb="242">
+      <t>ジュンバン</t>
+    </rPh>
+    <rPh sb="243" eb="245">
+      <t>ヒョウジ</t>
+    </rPh>
+    <rPh sb="247" eb="248">
+      <t>ホ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="8"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Yu Gothic"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
     </font>
     <font>
       <sz val="10"/>
@@ -726,7 +841,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,12 +851,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCCFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -757,97 +866,112 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
@@ -1138,442 +1262,512 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
     <col min="1" max="2" width="3.921875" style="2" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="51.84375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="4.4609375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.3046875" style="5" customWidth="1"/>
-    <col min="7" max="7" width="9.921875" style="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.15234375" style="15" customWidth="1"/>
-    <col min="9" max="9" width="9.23046875" style="5"/>
-    <col min="10" max="16384" width="9.23046875" style="1"/>
+    <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.3046875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.921875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="42.15234375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="9.23046875" style="5"/>
+    <col min="11" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="20"/>
-      <c r="B1" s="20"/>
-      <c r="C1" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="22"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="I1" s="24" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="50.6">
+    <row r="1" spans="1:10">
+      <c r="A1" s="19"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="21"/>
+      <c r="F1" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="I1" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="50.6">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="B3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="B3" s="6" t="s">
+      <c r="C4" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="B5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="B4" s="6" t="s">
+      <c r="C5" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="B6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="B5" s="6" t="s">
+      <c r="C6" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="B7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="B6" s="6" t="s">
+      <c r="C7" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="B8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="B7" s="6" t="s">
+      <c r="C8" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="B8" s="6" t="s">
+      <c r="C9" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="B10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="B9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="B10" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="C10" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="33.75">
+      <c r="B11" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="33.75">
       <c r="A12" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>42</v>
+      <c r="B12" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="33.75">
+        <v>19</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="33.75">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>42</v>
+      <c r="B13" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="101.2">
+    </row>
+    <row r="14" spans="1:10" ht="101.2">
       <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>42</v>
+      <c r="B14" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="50.6">
+      <c r="E14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="50.6">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>42</v>
+      <c r="B15" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H15" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="101.2">
+        <v>24</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="I15" s="18"/>
+    </row>
+    <row r="16" spans="1:10" ht="101.2">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>42</v>
+      <c r="B16" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>42</v>
+      <c r="B17" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="B18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>42</v>
+      <c r="E17" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="B18" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>42</v>
+      <c r="B19" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="67.45">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="50.6">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>42</v>
+      <c r="B20" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="50.6">
+        <v>17</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" s="35"/>
+    </row>
+    <row r="21" spans="1:10" ht="50.6">
       <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="50.6">
-      <c r="B22" s="31" t="s">
+      <c r="C21" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="101.2">
+      <c r="B22" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D22" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="F22" s="7"/>
-    </row>
-    <row r="23" spans="1:9" ht="33.75">
+      <c r="C22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="27">
+        <v>0.6</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="I22" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="J22" s="24" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="33.75">
       <c r="A23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="B23" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="134.9">
+      <c r="A24" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="33.75">
+      <c r="A25" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="134.9">
-      <c r="A24" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="9" t="s">
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="33.75">
+      <c r="A27" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G27" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G24" s="13" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="33.75">
-      <c r="A25" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="J27" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="118.05">
+      <c r="A28" s="10" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="33.75">
-      <c r="A27" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="B28" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="G27" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="I27" s="17" t="s">
+      <c r="E28" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I28" s="18" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="118.05">
-      <c r="A28" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="G28" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="H28" s="19" t="s">
+    <row r="29" spans="1:10" ht="33.75">
+      <c r="A29" s="23" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="33.75">
-      <c r="A29" s="25" t="s">
+      <c r="B29" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="J29" s="24" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="67.45">
+      <c r="A30" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="B29" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D29" s="18" t="s">
+      <c r="B30" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="30">
-        <v>0.5</v>
-      </c>
-      <c r="I29" s="26" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="67.45">
-      <c r="A30" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="B30" s="31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30" s="29" t="s">
+      <c r="E30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="J30" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="30">
-        <v>0.03</v>
+    </row>
+    <row r="31" spans="1:10" ht="118.05">
+      <c r="A31" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="31" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="7"/>
+  <phoneticPr fontId="8"/>
   <hyperlinks>
-    <hyperlink ref="I29" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
+    <hyperlink ref="J29" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
+    <hyperlink ref="J22" r:id="rId2" location="64" xr:uid="{52043B27-C4EC-4B5C-9326-B5A0D68D6A6B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support custom thumbnails for fixed-page bookmarks
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FF4C9A-A59C-4EDB-80F5-058FEF5AD40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD8EDB2-9BAA-46D5-A1AD-B237900BBBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="86">
   <si>
     <t>0</t>
     <phoneticPr fontId="8"/>
@@ -761,6 +761,108 @@
   </si>
   <si>
     <t>0</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>6d35f5cf8</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>M</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>FixedブクマのサムネをFixedしたページの画像にする。</t>
+    <rPh sb="24" eb="26">
+      <t>ガゾウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Bookmark.cs
+BookmarkCollection.cs
+BookmarkCollectionService.cs
+BookmarkFolderCollection.cs
+FolderCollection.cs
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>「ブックマーク」パネル内のフォルダーの中にサブフォルダーが存在する場合のCtrl + DとCtrl+Shift+Dの挙動がおかしい。
+この処理が実行されるパスは2系統ある。
+①「本棚」側がトリガーでAddToにたどり着く系統。
+②「メイン」側や「ブックマーク」側がトリガーでAddToにたどり着く系統。
+どっちも詳細調査が必要だが、特に②系統目があやしい。</t>
+    <rPh sb="11" eb="12">
+      <t>ナイ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>ナカ</t>
+    </rPh>
+    <rPh sb="29" eb="31">
+      <t>ソンザイ</t>
+    </rPh>
+    <rPh sb="33" eb="35">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="58" eb="60">
+      <t>キョドウ</t>
+    </rPh>
+    <rPh sb="69" eb="71">
+      <t>ショリ</t>
+    </rPh>
+    <rPh sb="72" eb="74">
+      <t>ジッコウ</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>ケイトウ</t>
+    </rPh>
+    <rPh sb="89" eb="91">
+      <t>ホンダナ</t>
+    </rPh>
+    <rPh sb="92" eb="93">
+      <t>ガワ</t>
+    </rPh>
+    <rPh sb="108" eb="109">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="110" eb="112">
+      <t>ケイトウ</t>
+    </rPh>
+    <rPh sb="120" eb="121">
+      <t>ガワ</t>
+    </rPh>
+    <rPh sb="130" eb="131">
+      <t>ガワ</t>
+    </rPh>
+    <rPh sb="146" eb="147">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="148" eb="150">
+      <t>ケイトウ</t>
+    </rPh>
+    <rPh sb="156" eb="158">
+      <t>ショウサイ</t>
+    </rPh>
+    <rPh sb="158" eb="160">
+      <t>チョウサ</t>
+    </rPh>
+    <rPh sb="161" eb="163">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <rPh sb="166" eb="167">
+      <t>トク</t>
+    </rPh>
+    <rPh sb="169" eb="171">
+      <t>ケイトウ</t>
+    </rPh>
+    <rPh sb="171" eb="172">
+      <t>メ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>N</t>
     <phoneticPr fontId="8"/>
   </si>
 </sst>
@@ -841,7 +943,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -851,6 +953,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE7FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -883,9 +991,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -896,9 +1001,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -922,9 +1024,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -934,24 +1033,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -973,8 +1063,26 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="9" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -985,6 +1093,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFE7FF"/>
       <color rgb="FFFFCCFF"/>
     </mruColors>
   </colors>
@@ -1262,163 +1371,161 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="2" width="3.921875" style="2" customWidth="1"/>
+    <col min="1" max="2" width="3.921875" style="31" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="51.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="43.3046875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="9.921875" style="13" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="42.15234375" style="14" customWidth="1"/>
+    <col min="6" max="6" width="37.61328125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.921875" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="42.15234375" style="12" customWidth="1"/>
     <col min="10" max="10" width="9.23046875" style="5"/>
     <col min="11" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="19"/>
-      <c r="B1" s="19"/>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="21"/>
-      <c r="F1" s="33" t="s">
+      <c r="D1" s="18"/>
+      <c r="F1" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="I1" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="19" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="50.6">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2" s="7" t="s">
+      <c r="C2" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="33.75">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="33.75">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H13" s="3" t="s">
@@ -1426,19 +1533,19 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="101.2">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>18</v>
       </c>
       <c r="H14" s="3" t="s">
@@ -1446,34 +1553,34 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="50.6">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="H15" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="I15" s="18"/>
+      <c r="I15" s="16"/>
     </row>
     <row r="16" spans="1:10" ht="101.2">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -1485,27 +1592,27 @@
       <c r="I16" s="3"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -1513,13 +1620,13 @@
       </c>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -1527,238 +1634,266 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="50.6">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="35"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" spans="1:10" ht="50.6">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="C21" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="31" t="s">
+      <c r="F21" s="25" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="101.2">
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" s="26" t="s">
+      <c r="C22" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="27">
+      <c r="E22" s="30">
         <v>0.6</v>
       </c>
-      <c r="F22" s="31" t="s">
+      <c r="F22" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="I22" s="31" t="s">
+      <c r="I22" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="J22" s="24" t="s">
+      <c r="J22" s="20" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="33.75">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="8" t="s">
+      <c r="C23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="134.9">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C24" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" s="8" t="s">
+      <c r="C24" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G24" s="12" t="s">
+      <c r="G24" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="33.75">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="8" t="s">
+      <c r="C25" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="33.75">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="8" t="s">
+      <c r="C27" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="G27" s="15" t="s">
+      <c r="G27" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="J27" s="16" t="s">
+      <c r="J27" s="14" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="118.05">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="28" t="s">
+      <c r="B28" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="C28" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="G28" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="I28" s="18" t="s">
+      <c r="I28" s="16" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="33.75">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="28" t="s">
+      <c r="B29" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="17" t="s">
+      <c r="C29" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="27">
+      <c r="E29" s="22">
         <v>0.5</v>
       </c>
-      <c r="J29" s="24" t="s">
+      <c r="J29" s="20" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="67.45">
-      <c r="A30" s="25" t="s">
+      <c r="A30" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="B30" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="32" t="s">
+      <c r="C30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F30" s="31" t="s">
+      <c r="F30" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="G30" s="30" t="s">
+      <c r="G30" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="J30" s="29" t="s">
+      <c r="J30" s="23" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="118.05">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="28" t="s">
+      <c r="B31" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="31" t="s">
+      <c r="C31" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="25" t="s">
         <v>78</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="G31" s="24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="D32" s="25" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="118.05">
+      <c r="A33" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="25" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Fix] Use bookshelf selection for multi-bookmark creation
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD8EDB2-9BAA-46D5-A1AD-B237900BBBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EEF54F-255F-44B5-BD9E-3D2259CD282B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="88">
   <si>
     <t>0</t>
     <phoneticPr fontId="8"/>
@@ -788,81 +788,94 @@
     <phoneticPr fontId="8"/>
   </si>
   <si>
-    <t>「ブックマーク」パネル内のフォルダーの中にサブフォルダーが存在する場合のCtrl + DとCtrl+Shift+Dの挙動がおかしい。
+    <t>N</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>b68bef0fb</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Bookmark.cs
+BookmarkCollection.cs
+BookmarkCollectionService.cs
+BookmarkFolderCollection.cs
+FolderItem.cs
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>「ブックマーク」内のどこかのフォルダーの中にサブフォルダーが存在する場合のCtrl + DとCtrl+Shift+Dの挙動がおかしい。
 この処理が実行されるパスは2系統ある。
 ①「本棚」側がトリガーでAddToにたどり着く系統。
 ②「メイン」側や「ブックマーク」側がトリガーでAddToにたどり着く系統。
 どっちも詳細調査が必要だが、特に②系統目があやしい。</t>
-    <rPh sb="11" eb="12">
+    <rPh sb="8" eb="9">
       <t>ナイ</t>
     </rPh>
-    <rPh sb="19" eb="20">
+    <rPh sb="20" eb="21">
       <t>ナカ</t>
     </rPh>
-    <rPh sb="29" eb="31">
+    <rPh sb="30" eb="32">
       <t>ソンザイ</t>
     </rPh>
-    <rPh sb="33" eb="35">
+    <rPh sb="34" eb="36">
       <t>バアイ</t>
     </rPh>
-    <rPh sb="58" eb="60">
+    <rPh sb="59" eb="61">
       <t>キョドウ</t>
     </rPh>
-    <rPh sb="69" eb="71">
+    <rPh sb="70" eb="72">
       <t>ショリ</t>
     </rPh>
-    <rPh sb="72" eb="74">
+    <rPh sb="73" eb="75">
       <t>ジッコウ</t>
     </rPh>
-    <rPh sb="81" eb="83">
+    <rPh sb="82" eb="84">
       <t>ケイトウ</t>
     </rPh>
-    <rPh sb="89" eb="91">
+    <rPh sb="90" eb="92">
       <t>ホンダナ</t>
     </rPh>
-    <rPh sb="92" eb="93">
+    <rPh sb="93" eb="94">
       <t>ガワ</t>
     </rPh>
-    <rPh sb="108" eb="109">
+    <rPh sb="109" eb="110">
       <t>ツ</t>
     </rPh>
-    <rPh sb="110" eb="112">
+    <rPh sb="111" eb="113">
       <t>ケイトウ</t>
     </rPh>
-    <rPh sb="120" eb="121">
+    <rPh sb="121" eb="122">
       <t>ガワ</t>
     </rPh>
-    <rPh sb="130" eb="131">
+    <rPh sb="131" eb="132">
       <t>ガワ</t>
     </rPh>
-    <rPh sb="146" eb="147">
+    <rPh sb="147" eb="148">
       <t>ツ</t>
     </rPh>
-    <rPh sb="148" eb="150">
+    <rPh sb="149" eb="151">
       <t>ケイトウ</t>
     </rPh>
-    <rPh sb="156" eb="158">
+    <rPh sb="157" eb="159">
       <t>ショウサイ</t>
     </rPh>
-    <rPh sb="158" eb="160">
+    <rPh sb="159" eb="161">
       <t>チョウサ</t>
     </rPh>
-    <rPh sb="161" eb="163">
+    <rPh sb="162" eb="164">
       <t>ヒツヨウ</t>
     </rPh>
-    <rPh sb="166" eb="167">
+    <rPh sb="167" eb="168">
       <t>トク</t>
     </rPh>
-    <rPh sb="169" eb="171">
+    <rPh sb="170" eb="172">
       <t>ケイトウ</t>
     </rPh>
-    <rPh sb="171" eb="172">
+    <rPh sb="172" eb="173">
       <t>メ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
-    <t>N</t>
     <phoneticPr fontId="8"/>
   </si>
 </sst>
@@ -1376,7 +1389,7 @@
   <cols>
     <col min="1" max="2" width="3.921875" style="31" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="51.84375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="56.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37.61328125" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.921875" style="11" bestFit="1" customWidth="1"/>
@@ -1877,7 +1890,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" ht="101.2">
       <c r="A32" s="34" t="s">
         <v>81</v>
       </c>
@@ -1887,13 +1900,22 @@
       <c r="D32" s="25" t="s">
         <v>82</v>
       </c>
+      <c r="E32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="118.05">
       <c r="A33" s="34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Feat] Enable clickable bookmark tags on bookshelf thumbnails to sync bookmark panel and support Enter folder navigation
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EEF54F-255F-44B5-BD9E-3D2259CD282B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63667D3E-F308-476B-B873-8BF415AE785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="91">
   <si>
     <t>0</t>
     <phoneticPr fontId="8"/>
@@ -875,6 +875,33 @@
     </rPh>
     <rPh sb="172" eb="173">
       <t>メ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>ea754c3a1</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>BookmarkCollectionService.cs
+CreateBookmarkCommand.cs
+FolderList.cs
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>既によく似た機能が本家バージョンにあったため、カスタマイズせず</t>
+    <rPh sb="0" eb="1">
+      <t>スデ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ニ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>キノウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ホンケ</t>
     </rPh>
     <phoneticPr fontId="8"/>
   </si>
@@ -1765,8 +1792,17 @@
       <c r="B26" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="C26" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="25" t="s">
         <v>47</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="23" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="33.75">
@@ -1897,6 +1933,9 @@
       <c r="B32" s="34" t="s">
         <v>79</v>
       </c>
+      <c r="C32" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="D32" s="25" t="s">
         <v>82</v>
       </c>
@@ -1910,12 +1949,27 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="118.05">
+    <row r="33" spans="1:7" ht="118.05">
       <c r="A33" s="34" t="s">
         <v>84</v>
       </c>
+      <c r="B33" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="D33" s="25" t="s">
         <v>87</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Feat] Rank bookshelf items by fixed bookmark count using star overlays
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63667D3E-F308-476B-B873-8BF415AE785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC2EF5A-5ABE-4156-8387-C1A4B61AC75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="98">
   <si>
     <t>0</t>
     <phoneticPr fontId="8"/>
@@ -890,7 +890,9 @@
     <phoneticPr fontId="8"/>
   </si>
   <si>
-    <t>既によく似た機能が本家バージョンにあったため、カスタマイズせず</t>
+    <t>既によく似た機能が本家バージョンにあったため、カスタマイズせず。
+代わりに「ブックマーク」でのキーバインドを少し変更する。
+Enterキーでフォルダーの中へ入る。</t>
     <rPh sb="0" eb="1">
       <t>スデ</t>
     </rPh>
@@ -903,6 +905,104 @@
     <rPh sb="9" eb="11">
       <t>ホンケ</t>
     </rPh>
+    <rPh sb="33" eb="34">
+      <t>カ</t>
+    </rPh>
+    <rPh sb="54" eb="55">
+      <t>スコ</t>
+    </rPh>
+    <rPh sb="56" eb="58">
+      <t>ヘンコウ</t>
+    </rPh>
+    <rPh sb="76" eb="77">
+      <t>ナカ</t>
+    </rPh>
+    <rPh sb="78" eb="79">
+      <t>ハイ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>016103053</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>ISearchBoxComponent.cs
+SearchBox.xaml
+SearchBox.xaml.cs
+SearchBoxModel.cs
+BookmarkFolderList.cs
+BookmarkListView.xaml
+FolderListBox.xaml
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>■虫眼鏡でルート検索
+■「Enter」キーでフォルダーの中へ入る
+■「本棚」のブクマ・タグをクリックすることにより、「ブックマーク」の対応するフォルダーを開く</t>
+    <rPh sb="1" eb="4">
+      <t>ムシメガネ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>ケンサク</t>
+    </rPh>
+    <rPh sb="28" eb="29">
+      <t>ナカ</t>
+    </rPh>
+    <rPh sb="30" eb="31">
+      <t>ハイ</t>
+    </rPh>
+    <rPh sb="35" eb="37">
+      <t>ホンダナ</t>
+    </rPh>
+    <rPh sb="67" eb="69">
+      <t>タイオウ</t>
+    </rPh>
+    <rPh sb="77" eb="78">
+      <t>ヒラ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>P</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>コンテキストメニューで「ブックマークの切り取り」を追加</t>
+    <rPh sb="19" eb="20">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="21" eb="22">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="25" eb="27">
+      <t>ツイカ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>URLもあたかも一つのファイルの様に扱い、Chrome等からのD&amp;D対応</t>
+    <rPh sb="8" eb="9">
+      <t>ヒト</t>
+    </rPh>
+    <rPh sb="16" eb="17">
+      <t>ヨウ</t>
+    </rPh>
+    <rPh sb="18" eb="19">
+      <t>アツカ</t>
+    </rPh>
+    <rPh sb="27" eb="28">
+      <t>トウ</t>
+    </rPh>
+    <rPh sb="34" eb="36">
+      <t>タイオウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t xml:space="preserve">FolderItem:UpdateOverLay( ) L452
+</t>
     <phoneticPr fontId="8"/>
   </si>
 </sst>
@@ -1079,9 +1179,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1123,6 +1220,9 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1411,17 +1511,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="2" width="3.921875" style="31" customWidth="1"/>
+    <col min="1" max="2" width="3.921875" style="30" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="56.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37.61328125" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.921875" style="11" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="42.15234375" style="12" customWidth="1"/>
-    <col min="10" max="10" width="9.23046875" style="5"/>
+    <col min="10" max="10" width="47.07421875" style="5" customWidth="1"/>
     <col min="11" max="16384" width="9.23046875" style="1"/>
   </cols>
   <sheetData>
@@ -1430,16 +1530,16 @@
         <v>39</v>
       </c>
       <c r="D1" s="18"/>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="26" t="s">
         <v>73</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="28" t="s">
+      <c r="H1" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="27" t="s">
         <v>75</v>
       </c>
       <c r="J1" s="19" t="s">
@@ -1447,10 +1547,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="50.6">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="34" t="s">
         <v>25</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1461,7 +1561,7 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="34" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -1469,7 +1569,7 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="34" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -1477,7 +1577,7 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="34" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1485,7 +1585,7 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1493,7 +1593,7 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -1501,7 +1601,7 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="34" t="s">
         <v>31</v>
       </c>
       <c r="C8" s="9" t="s">
@@ -1509,7 +1609,7 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -1517,7 +1617,7 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="34" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -1525,10 +1625,10 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -1536,10 +1636,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="33.75">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -1553,10 +1653,10 @@
       </c>
     </row>
     <row r="13" spans="1:10" ht="33.75">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -1573,10 +1673,10 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="101.2">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1593,10 +1693,10 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="50.6">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -1614,10 +1714,10 @@
       <c r="I15" s="16"/>
     </row>
     <row r="16" spans="1:10" ht="101.2">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C16" s="9" t="s">
@@ -1632,10 +1732,10 @@
       <c r="I16" s="3"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="33" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -1649,7 +1749,7 @@
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="33" t="s">
         <v>1</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -1660,10 +1760,10 @@
       </c>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -1674,10 +1774,10 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="50.6">
-      <c r="A20" s="31" t="s">
+      <c r="A20" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -1689,13 +1789,13 @@
       <c r="E20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="29"/>
+      <c r="H20" s="28"/>
     </row>
     <row r="21" spans="1:10" ht="50.6">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="35" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1707,12 +1807,12 @@
       <c r="E21" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F21" s="25" t="s">
+      <c r="F21" s="24" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="101.2">
-      <c r="B22" s="36" t="s">
+      <c r="B22" s="35" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="9" t="s">
@@ -1721,13 +1821,13 @@
       <c r="D22" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="29">
         <v>0.6</v>
       </c>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="I22" s="25" t="s">
+      <c r="I22" s="24" t="s">
         <v>72</v>
       </c>
       <c r="J22" s="20" t="s">
@@ -1735,10 +1835,10 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="33.75">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="9" t="s">
@@ -1752,7 +1852,7 @@
       <c r="A24" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="9" t="s">
@@ -1775,7 +1875,7 @@
       <c r="A25" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -1785,23 +1885,32 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" ht="134.9">
       <c r="A26" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="25" t="s">
+      <c r="D26" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J26" s="23" t="s">
+      <c r="F26" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="H26" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="J26" s="24" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1809,7 +1918,7 @@
       <c r="A27" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="36" t="s">
+      <c r="B27" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -1835,7 +1944,7 @@
       <c r="A28" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="36" t="s">
+      <c r="B28" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C28" s="9" t="s">
@@ -1847,7 +1956,7 @@
       <c r="E28" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F28" s="24" t="s">
         <v>56</v>
       </c>
       <c r="G28" s="13" t="s">
@@ -1858,10 +1967,10 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="33.75">
-      <c r="A29" s="32" t="s">
+      <c r="A29" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="9" t="s">
@@ -1870,106 +1979,125 @@
       <c r="D29" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="22">
-        <v>0.5</v>
+      <c r="E29" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H29" s="36" t="s">
+        <v>97</v>
       </c>
       <c r="J29" s="20" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="67.45">
-      <c r="A30" s="33" t="s">
+      <c r="A30" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="B30" s="36" t="s">
+      <c r="B30" s="35" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="26" t="s">
+      <c r="D30" s="25" t="s">
         <v>65</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F30" s="25" t="s">
+      <c r="F30" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="G30" s="24" t="s">
+      <c r="G30" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="J30" s="23" t="s">
+      <c r="J30" s="22" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="118.05">
-      <c r="A31" s="34" t="s">
+      <c r="A31" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="36" t="s">
+      <c r="B31" s="35" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D31" s="25" t="s">
+      <c r="D31" s="24" t="s">
         <v>78</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F31" s="25" t="s">
+      <c r="F31" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="G31" s="24" t="s">
+      <c r="G31" s="23" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="101.2">
-      <c r="A32" s="34" t="s">
+      <c r="A32" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="34" t="s">
+      <c r="B32" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="25" t="s">
+      <c r="D32" s="24" t="s">
         <v>82</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="25" t="s">
+      <c r="F32" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="G32" s="24" t="s">
+      <c r="G32" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="118.05">
-      <c r="A33" s="34" t="s">
+      <c r="A33" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="34" t="s">
+      <c r="B33" s="33" t="s">
         <v>79</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D33" s="25" t="s">
+      <c r="D33" s="24" t="s">
         <v>87</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="25" t="s">
+      <c r="F33" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="G33" s="24" t="s">
+      <c r="G33" s="23" t="s">
         <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="D35" s="24" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Feat] Continue Shift+Left/Right selection across thumbnail row boundaries
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC2EF5A-5ABE-4156-8387-C1A4B61AC75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650269F4-4B17-4F3D-AB37-C01D1004ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="114">
   <si>
     <t>0</t>
     <phoneticPr fontId="8"/>
@@ -489,31 +489,6 @@
     <phoneticPr fontId="8"/>
   </si>
   <si>
-    <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？</t>
-    <rPh sb="9" eb="10">
-      <t>カズ</t>
-    </rPh>
-    <rPh sb="16" eb="18">
-      <t>ホンダナ</t>
-    </rPh>
-    <rPh sb="20" eb="21">
-      <t>ホン</t>
-    </rPh>
-    <rPh sb="22" eb="24">
-      <t>ミギカタ</t>
-    </rPh>
-    <rPh sb="25" eb="27">
-      <t>ヒョウジ</t>
-    </rPh>
-    <rPh sb="31" eb="32">
-      <t>イロ</t>
-    </rPh>
-    <rPh sb="33" eb="34">
-      <t>カ</t>
-    </rPh>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
     <t>https://chatgpt.com/c/6a2f9616-be38-83e8-b9d9-edc6d1622263#12-1</t>
     <phoneticPr fontId="8"/>
   </si>
@@ -657,35 +632,6 @@
   <si>
     <t>FolderListBox.xaml.cs
 ListBoxThumbnailLoader.cs</t>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
-    <t>リセット
- _shiftSelectionAnchorIndex = -1;
- _shiftSelectionCurrentIndex = -1;
-■マウスで飛ぶ場合。
-■Shift + ← or Shift + →で選択範囲を開始。途中でShift + ↑の操作をしたときの選択範囲が異常</t>
-    <rPh sb="79" eb="80">
-      <t>ト</t>
-    </rPh>
-    <rPh sb="81" eb="83">
-      <t>バアイ</t>
-    </rPh>
-    <rPh sb="117" eb="119">
-      <t>トチュウ</t>
-    </rPh>
-    <rPh sb="130" eb="132">
-      <t>ソウサ</t>
-    </rPh>
-    <rPh sb="138" eb="140">
-      <t>センタク</t>
-    </rPh>
-    <rPh sb="140" eb="142">
-      <t>ハンイ</t>
-    </rPh>
-    <rPh sb="143" eb="145">
-      <t>イジョウ</t>
-    </rPh>
     <phoneticPr fontId="8"/>
   </si>
   <si>
@@ -1003,6 +949,150 @@
   <si>
     <t xml:space="preserve">FolderItem:UpdateOverLay( ) L452
 </t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>FolderItem.cs
+FolderListIcon.cs
+Generic.xaml</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>300afb0a6
+amended
+1807c3861</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>e50a1a24c</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>FolderItem.cs
+FolderListBox.xaml
+FolderListBox.xaml.cs</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>サムネにオーバーレイしてるタグがおおくなったら、(6つ以上)一番下に「…」ってだして、その「…」をクリックしたら残りのタグも含めた全体タグ表示できるようにしたいなぁ</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Q</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？→
+★の色から、♥の数でグレードを表すに変更</t>
+    <rPh sb="9" eb="10">
+      <t>カズ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>ホンダナ</t>
+    </rPh>
+    <rPh sb="20" eb="21">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t>ミギカタ</t>
+    </rPh>
+    <rPh sb="25" eb="27">
+      <t>ヒョウジ</t>
+    </rPh>
+    <rPh sb="31" eb="32">
+      <t>イロ</t>
+    </rPh>
+    <rPh sb="33" eb="34">
+      <t>カ</t>
+    </rPh>
+    <rPh sb="45" eb="46">
+      <t>イロ</t>
+    </rPh>
+    <rPh sb="51" eb="52">
+      <t>カズ</t>
+    </rPh>
+    <rPh sb="58" eb="59">
+      <t>アラワ</t>
+    </rPh>
+    <rPh sb="61" eb="63">
+      <t>ヘンコウ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>サムネの大きさが変えられなくなった</t>
+    <rPh sb="4" eb="5">
+      <t>オオ</t>
+    </rPh>
+    <rPh sb="8" eb="9">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>R</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>S</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>T</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>U</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>V</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>W</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Y</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>Z</t>
+    <phoneticPr fontId="8"/>
+  </si>
+  <si>
+    <t>リセット
+ _shiftSelectionAnchorIndex = -1;
+ _shiftSelectionCurrentIndex = -1;
+■マウスで飛ぶ場合。
+■Shift + ← or Shift + →で選択範囲を開始。途中でShift + ↑の操作をしたときの選択範囲が異常
+■#1832</t>
+    <rPh sb="79" eb="80">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>バアイ</t>
+    </rPh>
+    <rPh sb="117" eb="119">
+      <t>トチュウ</t>
+    </rPh>
+    <rPh sb="130" eb="132">
+      <t>ソウサ</t>
+    </rPh>
+    <rPh sb="138" eb="140">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="140" eb="142">
+      <t>ハンイ</t>
+    </rPh>
+    <rPh sb="143" eb="145">
+      <t>イジョウ</t>
+    </rPh>
     <phoneticPr fontId="8"/>
   </si>
 </sst>
@@ -1116,7 +1206,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1222,6 +1312,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1511,7 +1604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
     <col min="1" max="2" width="3.921875" style="30" customWidth="1"/>
@@ -1531,16 +1624,16 @@
       </c>
       <c r="D1" s="18"/>
       <c r="F1" s="26" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>51</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I1" s="27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J1" s="19" t="s">
         <v>59</v>
@@ -1629,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>40</v>
@@ -1640,7 +1733,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>40</v>
@@ -1657,7 +1750,7 @@
         <v>3</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>40</v>
@@ -1677,7 +1770,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>40</v>
@@ -1697,7 +1790,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>40</v>
@@ -1718,7 +1811,7 @@
         <v>6</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>40</v>
@@ -1764,7 +1857,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>40</v>
@@ -1778,7 +1871,7 @@
         <v>9</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>40</v>
@@ -1811,7 +1904,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="101.2">
+    <row r="22" spans="1:10" ht="118.05">
       <c r="B22" s="35" t="s">
         <v>1</v>
       </c>
@@ -1819,19 +1912,19 @@
         <v>40</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E22" s="29">
         <v>0.6</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="J22" s="20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="33.75">
@@ -1839,7 +1932,7 @@
         <v>11</v>
       </c>
       <c r="B23" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C23" s="9" t="s">
         <v>40</v>
@@ -1853,7 +1946,7 @@
         <v>37</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>40</v>
@@ -1876,7 +1969,7 @@
         <v>41</v>
       </c>
       <c r="B25" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C25" s="9" t="s">
         <v>40</v>
@@ -1890,7 +1983,7 @@
         <v>44</v>
       </c>
       <c r="B26" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>40</v>
@@ -1902,16 +1995,16 @@
         <v>18</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G26" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="H26" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="H26" s="36" t="s">
-        <v>93</v>
-      </c>
       <c r="J26" s="24" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="33.75">
@@ -1919,7 +2012,7 @@
         <v>45</v>
       </c>
       <c r="B27" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>40</v>
@@ -1945,7 +2038,7 @@
         <v>49</v>
       </c>
       <c r="B28" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>40</v>
@@ -1966,58 +2059,64 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="33.75">
+    <row r="29" spans="1:10" ht="50.6">
       <c r="A29" s="31" t="s">
         <v>61</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="15" t="s">
-        <v>62</v>
+      <c r="D29" s="24" t="s">
+        <v>102</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="F29" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="G29" s="37" t="s">
+        <v>97</v>
+      </c>
       <c r="H29" s="36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="J29" s="20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="67.45">
       <c r="A30" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="25" t="s">
         <v>64</v>
-      </c>
-      <c r="B30" s="35" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="25" t="s">
-        <v>65</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F30" s="24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J30" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="118.05">
       <c r="A31" s="33" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B31" s="35" t="s">
         <v>0</v>
@@ -2026,78 +2125,150 @@
         <v>40</v>
       </c>
       <c r="D31" s="24" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F31" s="24" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="101.2">
       <c r="A32" s="33" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F32" s="24" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="118.05">
       <c r="A33" s="33" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D33" s="24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F33" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="50.6">
       <c r="A34" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="G34" s="23" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="50.6">
+      <c r="A35" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="B35" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="B34" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="D34" s="24" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="D35" s="24" t="s">
-        <v>96</v>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" s="24" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="33" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="33" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="33" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="33" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="33" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="33" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="33" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[WIP] Introduce bookshelf thumbnail settings popup with direct config bindings
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650269F4-4B17-4F3D-AB37-C01D1004ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE40DBB-E370-438B-A8C3-B5FCF624A848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11055" yWindow="19686" windowWidth="24006" windowHeight="19723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,74 +25,74 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="121">
   <si>
     <t>0</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>9</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>B</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>ルート検索(トグル)の機能追加</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>検索窓にキーワードを打ち込んだら、currentフォルダーから下を対象に検索を開始するのやけど、ルート検索にしたら、ルートに設定してあるフォルダー(「本棚」なら、ホーム・ディレクトリあたりが適任。「ブックマーク」なら、ルート)からの検索になる仕様追加変更の検討。</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>NeeView内削除 → 関連ブクマ削除</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>ブックマーク・リングの再設定追加機能</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>メインビュー → ブックマークフォルダー D&amp;D登録</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>「本棚」パネルのタイトルバーにブックタイトルを表示。
@@ -109,14 +109,14 @@
     <rPh sb="55" eb="57">
       <t>ドウキ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>完了</t>
     <rPh sb="0" eb="2">
       <t>カンリョウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>サムネ・アイコン表示モードでの長すぎるファイル名の最後尾からちょい手前を省略する機能</t>
@@ -135,7 +135,7 @@
     <rPh sb="36" eb="38">
       <t>ショウリャク</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FolderTreeViewで「新しいフォルダー」コンテキストメニューをクリックしたときの挙動改善</t>
@@ -148,7 +148,7 @@
     <rPh sb="47" eb="49">
       <t>カイゼン</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■ブックマークをブクマ・フォルダーからブクマ・フォルダーへD&amp;Dでポイしたら、ポイした先にブクマは移動。
@@ -174,12 +174,12 @@
     <rPh sb="110" eb="111">
       <t>サキ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■ TreeView→ListBox同期経路を探索
 ■ListBox表示切替の正式ルート</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■ブックマークのコピーと貼り付け
@@ -196,7 +196,7 @@
     <rPh sb="38" eb="40">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>「ブックマーク」パネルのに「←→」ボタンを追加。
@@ -216,59 +216,59 @@
     <rPh sb="61" eb="63">
       <t>デキ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Bookmark.OpenPageMode（Resume / Fixed）をちゃんと動かすために、NeeViewの「本を開く流れ」を逆流調査してた。</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>private void FolderList_KeyDown(object? sender, KeyEventArgs e)</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>いまの設計では「本棚」パネルも「ページ」パネルもサムネ表示したときのサムネサイズはどちらも同じサイズで縛られてる。</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>C</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Ctrl + Shift + Dで「ブックマーク」パネルでSelectedなフォルダーに固定ページブクマを作成する</t>
@@ -278,19 +278,19 @@
     <rPh sb="53" eb="55">
       <t>サクセイ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>AI</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>〇</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>D</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>パネルをフローティングにしたときに、ショートカットキーで各パネルへフォーカスしてアクティブな状態にしたい。</t>
@@ -300,7 +300,7 @@
     <rPh sb="46" eb="48">
       <t>ジョウタイ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■「←→」キー打鍵だけでサムネ表示時のフォーカス・ブック移動を最初から最後までシームレスに移動できるようにする
@@ -335,15 +335,15 @@
     <rPh sb="67" eb="68">
       <t>カエ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>F</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>G</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>複数ファイルのCtrl+DとCtrl+Shift+Dの動作が単一ファイルしか操作されてなかった。</t>
@@ -359,7 +359,7 @@
     <rPh sb="38" eb="40">
       <t>ソウサ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>第一ホームと第二ホーム、第三ホームまでアイコン化</t>
@@ -375,7 +375,7 @@
     <rPh sb="23" eb="24">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>★印を固定ページブックマークの印として使えないか？</t>
@@ -391,19 +391,19 @@
     <rPh sb="19" eb="20">
       <t>ツカ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>H</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>5fdf7a0aa</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Git Commit</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>BookControl.cs
@@ -414,15 +414,15 @@
 ToggleBookmarkCommand.cs
 FolderListBox.xaml.cs
 BookAccessor.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>7640e4cc9</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>b4dc93aa4</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>make-links.ps1の運用を開始する</t>
@@ -432,7 +432,7 @@
     <rPh sb="18" eb="20">
       <t>カイシ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>BookmarkCollectionService.cs
@@ -442,12 +442,12 @@
 FolderListIcon.cs
 Colors.xaml
 NeeViewProjects.xlsx</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>CreateBookmarkCommand.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t xml:space="preserve">★のアイコンをクリックしたときの動作を追加する。
@@ -458,14 +458,14 @@
     <rPh sb="19" eb="21">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>その他</t>
     <rPh sb="2" eb="3">
       <t>タ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■本家からの返事。
@@ -482,19 +482,19 @@
     <rPh sb="26" eb="27">
       <t>オ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>J</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>https://chatgpt.com/c/6a2f9616-be38-83e8-b9d9-edc6d1622263#12-1</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>K</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>「本棚」でサムネの画像を指定するコンテキストメニューを実行したところ、不具合発生。
@@ -544,7 +544,7 @@
     <rPh sb="93" eb="95">
       <t>ハンエイホンダナヒョウジヒョウジドウキ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>行の一番端、右端でも左端でも、そこでShiftを押しながら、←→キーを叩いたら、次の行(下の段)、または前の行(上の段)に選択状態を維持したままカーソルが動いた。</t>
@@ -605,11 +605,11 @@
     <rPh sb="77" eb="78">
       <t>ウゴ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Cache.dbの存在を知る</t>
@@ -619,20 +619,20 @@
     <rPh sb="12" eb="13">
       <t>シ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>7ca3c5ebb</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FolderListBox.xaml.cs
 ListBoxThumbnailLoader.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>対象ファイル。関数。</t>
@@ -642,7 +642,7 @@
     <rPh sb="7" eb="9">
       <t>カンスウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>取り組み内容</t>
@@ -655,7 +655,7 @@
     <rPh sb="4" eb="6">
       <t>ナイヨウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>次回の課題</t>
@@ -665,15 +665,15 @@
     <rPh sb="3" eb="5">
       <t>カダイ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>https://chatgpt.com/c/6a2fc982-dc44-83ee-8d8d-af34bf9343d3#64</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>L</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>ファイルのファイル名によるソート順についての改善。
@@ -703,26 +703,26 @@
     <rPh sb="247" eb="248">
       <t>ホ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>6d35f5cf8</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>M</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FixedブクマのサムネをFixedしたページの画像にする。</t>
     <rPh sb="24" eb="26">
       <t>ガゾウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Bookmark.cs
@@ -731,15 +731,15 @@
 BookmarkFolderCollection.cs
 FolderCollection.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>N</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>b68bef0fb</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Bookmark.cs
@@ -748,7 +748,7 @@
 BookmarkFolderCollection.cs
 FolderItem.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>「ブックマーク」内のどこかのフォルダーの中にサブフォルダーが存在する場合のCtrl + DとCtrl+Shift+Dの挙動がおかしい。
@@ -822,18 +822,18 @@
     <rPh sb="172" eb="173">
       <t>メ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>ea754c3a1</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>BookmarkCollectionService.cs
 CreateBookmarkCommand.cs
 FolderList.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>既によく似た機能が本家バージョンにあったため、カスタマイズせず。
@@ -866,11 +866,11 @@
     <rPh sb="78" eb="79">
       <t>ハイ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>016103053</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>ISearchBoxComponent.cs
@@ -881,7 +881,7 @@
 BookmarkListView.xaml
 FolderListBox.xaml
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>■虫眼鏡でルート検索
@@ -908,11 +908,11 @@
     <rPh sb="77" eb="78">
       <t>ヒラ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>P</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>コンテキストメニューで「ブックマークの切り取り」を追加</t>
@@ -925,7 +925,7 @@
     <rPh sb="25" eb="27">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>URLもあたかも一つのファイルの様に扱い、Chrome等からのD&amp;D対応</t>
@@ -944,42 +944,42 @@
     <rPh sb="34" eb="36">
       <t>タイオウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t xml:space="preserve">FolderItem:UpdateOverLay( ) L452
 </t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FolderItem.cs
 FolderListIcon.cs
 Generic.xaml</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>300afb0a6
 amended
 1807c3861</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>e50a1a24c</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>FolderItem.cs
 FolderListBox.xaml
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>サムネにオーバーレイしてるタグがおおくなったら、(6つ以上)一番下に「…」ってだして、その「…」をクリックしたら残りのタグも含めた全体タグ表示できるようにしたいなぁ</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Q</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？→
@@ -1017,53 +1017,43 @@
     <rPh sb="61" eb="63">
       <t>ヘンコウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
-  </si>
-  <si>
-    <t>サムネの大きさが変えられなくなった</t>
-    <rPh sb="4" eb="5">
-      <t>オオ</t>
-    </rPh>
-    <rPh sb="8" eb="9">
-      <t>カ</t>
-    </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>R</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>S</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>T</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>U</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>V</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>W</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>X</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Y</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>Z</t>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
   </si>
   <si>
     <t>リセット
@@ -1093,20 +1083,75 @@
     <rPh sb="143" eb="145">
       <t>イジョウ</t>
     </rPh>
-    <phoneticPr fontId="8"/>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>ff5cbea85</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>FolderItem.cs
+FolderListBox.xaml
+FolderListBox.xaml.cs
+PanelListTextTools.cs</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>パネル毎にサムネの大きさを変える。</t>
+    <rPh sb="3" eb="4">
+      <t>ゴト</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>オオ</t>
+    </rPh>
+    <rPh sb="13" eb="14">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>1</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>2</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>c6d61eef6 (master)
+71a48c93c (master)</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>ce74d2bef (wip)</t>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>続き</t>
+    <rPh sb="0" eb="1">
+      <t>ツヅ</t>
+    </rPh>
+    <phoneticPr fontId="9"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Yu Gothic"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1204,118 +1249,133 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1604,10 +1664,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="2" width="3.921875" style="30" customWidth="1"/>
+    <col min="1" max="2" width="3.921875" style="29" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="56.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
@@ -1623,16 +1683,16 @@
         <v>39</v>
       </c>
       <c r="D1" s="18"/>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="25" t="s">
         <v>71</v>
       </c>
       <c r="G1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="I1" s="26" t="s">
         <v>73</v>
       </c>
       <c r="J1" s="19" t="s">
@@ -1640,10 +1700,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="50.6">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="33" t="s">
         <v>25</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1654,7 +1714,7 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="33" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -1662,7 +1722,7 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="33" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -1670,7 +1730,7 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="33" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1678,7 +1738,7 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="33" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1686,7 +1746,7 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="B7" s="34" t="s">
+      <c r="B7" s="33" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -1694,7 +1754,7 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="33" t="s">
         <v>31</v>
       </c>
       <c r="C8" s="9" t="s">
@@ -1702,7 +1762,7 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="33" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -1710,7 +1770,7 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="B10" s="34" t="s">
+      <c r="B10" s="33" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -1718,21 +1778,21 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="33.75">
-      <c r="A12" s="30" t="s">
+    <row r="12" spans="1:10" ht="67.45">
+      <c r="A12" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -1744,12 +1804,18 @@
       <c r="E12" s="8" t="s">
         <v>18</v>
       </c>
+      <c r="F12" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="G12" s="38" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="13" spans="1:10" ht="33.75">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -1766,10 +1832,10 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="101.2">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1786,10 +1852,10 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="50.6">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -1807,10 +1873,10 @@
       <c r="I15" s="16"/>
     </row>
     <row r="16" spans="1:10" ht="101.2">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C16" s="9" t="s">
@@ -1825,10 +1891,10 @@
       <c r="I16" s="3"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="32" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -1842,7 +1908,7 @@
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="32" t="s">
         <v>1</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -1853,10 +1919,10 @@
       </c>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -1867,10 +1933,10 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="50.6">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="33" t="s">
+      <c r="B20" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -1882,13 +1948,13 @@
       <c r="E20" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="H20" s="28"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" spans="1:10" ht="50.6">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="34" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1905,7 +1971,7 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="118.05">
-      <c r="B22" s="35" t="s">
+      <c r="B22" s="34" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="9" t="s">
@@ -1914,24 +1980,24 @@
       <c r="D22" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="28">
         <v>0.6</v>
       </c>
       <c r="F22" s="24" t="s">
         <v>69</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J22" s="20" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="33.75">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C23" s="9" t="s">
@@ -1945,7 +2011,7 @@
       <c r="A24" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="35" t="s">
+      <c r="B24" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C24" s="9" t="s">
@@ -1968,7 +2034,7 @@
       <c r="A25" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="35" t="s">
+      <c r="B25" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C25" s="9" t="s">
@@ -1982,7 +2048,7 @@
       <c r="A26" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="35" t="s">
+      <c r="B26" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C26" s="9" t="s">
@@ -2000,7 +2066,7 @@
       <c r="G26" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="36" t="s">
+      <c r="H26" s="35" t="s">
         <v>91</v>
       </c>
       <c r="J26" s="24" t="s">
@@ -2011,7 +2077,7 @@
       <c r="A27" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -2037,7 +2103,7 @@
       <c r="A28" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B28" s="35" t="s">
+      <c r="B28" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C28" s="9" t="s">
@@ -2060,10 +2126,10 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="50.6">
-      <c r="A29" s="31" t="s">
+      <c r="A29" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C29" s="9" t="s">
@@ -2078,10 +2144,10 @@
       <c r="F29" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="G29" s="37" t="s">
+      <c r="G29" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="H29" s="36" t="s">
+      <c r="H29" s="35" t="s">
         <v>95</v>
       </c>
       <c r="J29" s="20" t="s">
@@ -2089,16 +2155,16 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="67.45">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="35" t="s">
+      <c r="B30" s="34" t="s">
         <v>66</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="25" t="s">
+      <c r="D30" s="21" t="s">
         <v>64</v>
       </c>
       <c r="E30" s="8" t="s">
@@ -2115,10 +2181,10 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="118.05">
-      <c r="A31" s="33" t="s">
+      <c r="A31" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B31" s="35" t="s">
+      <c r="B31" s="34" t="s">
         <v>0</v>
       </c>
       <c r="C31" s="9" t="s">
@@ -2138,10 +2204,10 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="101.2">
-      <c r="A32" s="33" t="s">
+      <c r="A32" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="33" t="s">
+      <c r="B32" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C32" s="9" t="s">
@@ -2160,11 +2226,11 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="118.05">
-      <c r="A33" s="33" t="s">
+    <row r="33" spans="1:8" ht="118.05">
+      <c r="A33" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C33" s="9" t="s">
@@ -2183,11 +2249,11 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="50.6">
-      <c r="A34" s="33" t="s">
+    <row r="34" spans="1:8" ht="50.6">
+      <c r="A34" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="33" t="s">
+      <c r="B34" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C34" s="9" t="s">
@@ -2206,11 +2272,11 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="50.6">
-      <c r="A35" s="33" t="s">
+    <row r="35" spans="1:8" ht="50.6">
+      <c r="A35" s="32" t="s">
         <v>101</v>
       </c>
-      <c r="B35" s="33" t="s">
+      <c r="B35" s="32" t="s">
         <v>77</v>
       </c>
       <c r="C35" s="9" t="s">
@@ -2220,59 +2286,96 @@
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="33" t="s">
-        <v>104</v>
+    <row r="36" spans="1:8">
+      <c r="A36" s="32" t="s">
+        <v>103</v>
       </c>
       <c r="D36" s="24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="33" t="s">
+    <row r="37" spans="1:8">
+      <c r="A37" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="H37" s="41" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="33.75">
+      <c r="A38" s="1"/>
+      <c r="B38" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" s="42" t="s">
+        <v>120</v>
+      </c>
+      <c r="H38" s="37" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="1"/>
+      <c r="B39" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D39" s="42" t="s">
+        <v>120</v>
+      </c>
+      <c r="H39" s="37"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="32" t="s">
         <v>105</v>
       </c>
-      <c r="D37" s="24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="33" t="s">
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="32" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="33" t="s">
+    <row r="42" spans="1:8">
+      <c r="A42" s="32" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="33" t="s">
+    <row r="43" spans="1:8">
+      <c r="A43" s="32" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="33" t="s">
+    <row r="44" spans="1:8">
+      <c r="A44" s="32" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
-      <c r="A42" s="33" t="s">
+    <row r="45" spans="1:8">
+      <c r="A45" s="32" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
-      <c r="A43" s="33" t="s">
+    <row r="46" spans="1:8">
+      <c r="A46" s="32" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="44" spans="1:7">
-      <c r="A44" s="33" t="s">
-        <v>112</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="8"/>
+  <phoneticPr fontId="9"/>
   <hyperlinks>
     <hyperlink ref="J29" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
     <hyperlink ref="J22" r:id="rId2" location="64" xr:uid="{52043B27-C4EC-4B5C-9326-B5A0D68D6A6B}"/>

</xml_diff>

<commit_message>
[Feat] Complete separation of bookshelf and bookmark thumbnail settings
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE40DBB-E370-438B-A8C3-B5FCF624A848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B655BD2D-461B-4C70-9004-E3A007AE146B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="122">
   <si>
     <t>0</t>
     <phoneticPr fontId="9"/>
@@ -1131,6 +1131,10 @@
     <rPh sb="0" eb="1">
       <t>ツヅ</t>
     </rPh>
+    <phoneticPr fontId="9"/>
+  </si>
+  <si>
+    <t>d35ef5042 (master)</t>
     <phoneticPr fontId="9"/>
   </si>
 </sst>
@@ -1664,7 +1668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
     <col min="1" max="2" width="3.921875" style="29" customWidth="1"/>
@@ -2337,40 +2341,55 @@
       <c r="D39" s="42" t="s">
         <v>120</v>
       </c>
-      <c r="H39" s="37"/>
+      <c r="H39" s="37" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="32" t="s">
-        <v>105</v>
-      </c>
+      <c r="A40" s="1"/>
+      <c r="B40" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D40" s="42" t="s">
+        <v>120</v>
+      </c>
+      <c r="H40" s="37"/>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="32" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" s="32" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" s="32" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" s="32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="32" t="s">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[WIP] Prototype bookmark folder alias
</commit_message>
<xml_diff>
--- a/docs/NeeViewProjects.xlsx
+++ b/docs/NeeViewProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Test\NeeView\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B655BD2D-461B-4C70-9004-E3A007AE146B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51BCF54-23CD-4FA2-AA3E-72A59F91FD1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10991" yWindow="19650" windowWidth="24006" windowHeight="19722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,74 +25,74 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="131">
   <si>
     <t>0</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>9</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>A</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>B</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ルート検索(トグル)の機能追加</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>検索窓にキーワードを打ち込んだら、currentフォルダーから下を対象に検索を開始するのやけど、ルート検索にしたら、ルートに設定してあるフォルダー(「本棚」なら、ホーム・ディレクトリあたりが適任。「ブックマーク」なら、ルート)からの検索になる仕様追加変更の検討。</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>NeeView内削除 → 関連ブクマ削除</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ブックマーク・リングの再設定追加機能</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>メインビュー → ブックマークフォルダー D&amp;D登録</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>「本棚」パネルのタイトルバーにブックタイトルを表示。
@@ -109,14 +109,14 @@
     <rPh sb="55" eb="57">
       <t>ドウキ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>完了</t>
     <rPh sb="0" eb="2">
       <t>カンリョウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>サムネ・アイコン表示モードでの長すぎるファイル名の最後尾からちょい手前を省略する機能</t>
@@ -135,7 +135,7 @@
     <rPh sb="36" eb="38">
       <t>ショウリャク</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderTreeViewで「新しいフォルダー」コンテキストメニューをクリックしたときの挙動改善</t>
@@ -148,7 +148,7 @@
     <rPh sb="47" eb="49">
       <t>カイゼン</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■ブックマークをブクマ・フォルダーからブクマ・フォルダーへD&amp;Dでポイしたら、ポイした先にブクマは移動。
@@ -174,12 +174,12 @@
     <rPh sb="110" eb="111">
       <t>サキ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■ TreeView→ListBox同期経路を探索
 ■ListBox表示切替の正式ルート</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■ブックマークのコピーと貼り付け
@@ -196,7 +196,7 @@
     <rPh sb="38" eb="40">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>「ブックマーク」パネルのに「←→」ボタンを追加。
@@ -216,59 +216,59 @@
     <rPh sb="61" eb="63">
       <t>デキ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>3</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>5</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>6</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>7</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>8</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Bookmark.OpenPageMode（Resume / Fixed）をちゃんと動かすために、NeeViewの「本を開く流れ」を逆流調査してた。</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>private void FolderList_KeyDown(object? sender, KeyEventArgs e)</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>いまの設計では「本棚」パネルも「ページ」パネルもサムネ表示したときのサムネサイズはどちらも同じサイズで縛られてる。</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>C</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Ctrl + Shift + Dで「ブックマーク」パネルでSelectedなフォルダーに固定ページブクマを作成する</t>
@@ -278,19 +278,19 @@
     <rPh sb="53" eb="55">
       <t>サクセイ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>AI</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>〇</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>D</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>パネルをフローティングにしたときに、ショートカットキーで各パネルへフォーカスしてアクティブな状態にしたい。</t>
@@ -300,7 +300,7 @@
     <rPh sb="46" eb="48">
       <t>ジョウタイ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■「←→」キー打鍵だけでサムネ表示時のフォーカス・ブック移動を最初から最後までシームレスに移動できるようにする
@@ -335,15 +335,15 @@
     <rPh sb="67" eb="68">
       <t>カエ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>F</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>G</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>複数ファイルのCtrl+DとCtrl+Shift+Dの動作が単一ファイルしか操作されてなかった。</t>
@@ -359,7 +359,7 @@
     <rPh sb="38" eb="40">
       <t>ソウサ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>第一ホームと第二ホーム、第三ホームまでアイコン化</t>
@@ -375,7 +375,7 @@
     <rPh sb="23" eb="24">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>★印を固定ページブックマークの印として使えないか？</t>
@@ -391,19 +391,19 @@
     <rPh sb="19" eb="20">
       <t>ツカ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>H</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>5fdf7a0aa</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Git Commit</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>BookControl.cs
@@ -414,15 +414,15 @@
 ToggleBookmarkCommand.cs
 FolderListBox.xaml.cs
 BookAccessor.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>7640e4cc9</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>b4dc93aa4</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>make-links.ps1の運用を開始する</t>
@@ -432,7 +432,7 @@
     <rPh sb="18" eb="20">
       <t>カイシ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>BookmarkCollectionService.cs
@@ -442,12 +442,12 @@
 FolderListIcon.cs
 Colors.xaml
 NeeViewProjects.xlsx</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>CreateBookmarkCommand.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t xml:space="preserve">★のアイコンをクリックしたときの動作を追加する。
@@ -458,14 +458,14 @@
     <rPh sb="19" eb="21">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>その他</t>
     <rPh sb="2" eb="3">
       <t>タ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■本家からの返事。
@@ -482,19 +482,19 @@
     <rPh sb="26" eb="27">
       <t>オ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>J</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>https://chatgpt.com/c/6a2f9616-be38-83e8-b9d9-edc6d1622263#12-1</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>K</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>「本棚」でサムネの画像を指定するコンテキストメニューを実行したところ、不具合発生。
@@ -544,7 +544,7 @@
     <rPh sb="93" eb="95">
       <t>ハンエイホンダナヒョウジヒョウジドウキ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>行の一番端、右端でも左端でも、そこでShiftを押しながら、←→キーを叩いたら、次の行(下の段)、または前の行(上の段)に選択状態を維持したままカーソルが動いた。</t>
@@ -605,11 +605,11 @@
     <rPh sb="77" eb="78">
       <t>ウゴ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Cache.dbの存在を知る</t>
@@ -619,20 +619,20 @@
     <rPh sb="12" eb="13">
       <t>シ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>7ca3c5ebb</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderListBox.xaml.cs
 ListBoxThumbnailLoader.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>対象ファイル。関数。</t>
@@ -642,7 +642,7 @@
     <rPh sb="7" eb="9">
       <t>カンスウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>取り組み内容</t>
@@ -655,7 +655,7 @@
     <rPh sb="4" eb="6">
       <t>ナイヨウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>次回の課題</t>
@@ -665,15 +665,15 @@
     <rPh sb="3" eb="5">
       <t>カダイ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>https://chatgpt.com/c/6a2fc982-dc44-83ee-8d8d-af34bf9343d3#64</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>L</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ファイルのファイル名によるソート順についての改善。
@@ -703,26 +703,26 @@
     <rPh sb="247" eb="248">
       <t>ホ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>0</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>6d35f5cf8</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>M</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FixedブクマのサムネをFixedしたページの画像にする。</t>
     <rPh sb="24" eb="26">
       <t>ガゾウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Bookmark.cs
@@ -731,15 +731,15 @@
 BookmarkFolderCollection.cs
 FolderCollection.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>N</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>b68bef0fb</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Bookmark.cs
@@ -748,7 +748,7 @@
 BookmarkFolderCollection.cs
 FolderItem.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>「ブックマーク」内のどこかのフォルダーの中にサブフォルダーが存在する場合のCtrl + DとCtrl+Shift+Dの挙動がおかしい。
@@ -822,18 +822,18 @@
     <rPh sb="172" eb="173">
       <t>メ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ea754c3a1</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>BookmarkCollectionService.cs
 CreateBookmarkCommand.cs
 FolderList.cs
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>既によく似た機能が本家バージョンにあったため、カスタマイズせず。
@@ -866,11 +866,11 @@
     <rPh sb="78" eb="79">
       <t>ハイ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>016103053</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ISearchBoxComponent.cs
@@ -881,7 +881,7 @@
 BookmarkListView.xaml
 FolderListBox.xaml
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>■虫眼鏡でルート検索
@@ -908,11 +908,11 @@
     <rPh sb="77" eb="78">
       <t>ヒラ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>P</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>コンテキストメニューで「ブックマークの切り取り」を追加</t>
@@ -925,7 +925,7 @@
     <rPh sb="25" eb="27">
       <t>ツイカ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>URLもあたかも一つのファイルの様に扱い、Chrome等からのD&amp;D対応</t>
@@ -944,42 +944,42 @@
     <rPh sb="34" eb="36">
       <t>タイオウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t xml:space="preserve">FolderItem:UpdateOverLay( ) L452
 </t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderItem.cs
 FolderListIcon.cs
 Generic.xaml</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>300afb0a6
 amended
 1807c3861</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>e50a1a24c</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderItem.cs
 FolderListBox.xaml
 FolderListBox.xaml.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>サムネにオーバーレイしてるタグがおおくなったら、(6つ以上)一番下に「…」ってだして、その「…」をクリックしたら残りのタグも含めた全体タグ表示できるようにしたいなぁ</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Q</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Fixedブクマの数によって、「本棚」の本の右肩に表示する★の色を変えられないか？→
@@ -1017,43 +1017,43 @@
     <rPh sb="61" eb="63">
       <t>ヘンコウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>R</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>S</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>T</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>U</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>V</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>W</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>X</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Y</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>Z</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>リセット
@@ -1083,18 +1083,18 @@
     <rPh sb="143" eb="145">
       <t>イジョウ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ff5cbea85</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>FolderItem.cs
 FolderListBox.xaml
 FolderListBox.xaml.cs
 PanelListTextTools.cs</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>パネル毎にサムネの大きさを変える。</t>
@@ -1107,48 +1107,232 @@
     <rPh sb="13" eb="14">
       <t>カ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>1</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>2</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>c6d61eef6 (master)
 71a48c93c (master)</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>ce74d2bef (wip)</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>続き</t>
     <rPh sb="0" eb="1">
       <t>ツヅ</t>
     </rPh>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>d35ef5042 (master)</t>
-    <phoneticPr fontId="9"/>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>3</t>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>PanelsConfig.cs
+SettingPagePanels.cs
+BookmarkListView.xaml
+BookmarkListView.xaml.cs
+BookmarkThumbnailSettingPopup.xaml
+BookmarkThumbnailSettingPopup.xaml.cs
+BookshelfThumbnailSettingPopup.xaml
+BookshelfThumbnailSettingPopup.xaml.cs
+FolderListBox.xaml
+FolderListBox.xaml.cs
+FolderListBoxViewModel.cs
+FolderListView.xaml
+FolderListView.xaml.cs
+PanelListTextTools.cs
+PanelListThumbnailImage.cs
+NeeViewProjects.xlsx</t>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>6caa7d408 (最終, master)</t>
+    <rPh sb="11" eb="13">
+      <t>サイシュウ</t>
+    </rPh>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>ブックマークでフォルダーのエリアスを作る。</t>
+    <rPh sb="18" eb="19">
+      <t>ツク</t>
+    </rPh>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>←、→、Shift押しながらの←、→、Ctrl押しながら←、→、Ctrl+Shift押しながらの←、→全部の条件で右端、左端に到達したときの段またぎ(現在の段から、上段最後尾にワープ移動、下段最前にワープ移動)</t>
+    <rPh sb="9" eb="10">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="23" eb="24">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="42" eb="43">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="51" eb="53">
+      <t>ゼンブ</t>
+    </rPh>
+    <rPh sb="54" eb="56">
+      <t>ジョウケン</t>
+    </rPh>
+    <rPh sb="57" eb="59">
+      <t>ミギハジ</t>
+    </rPh>
+    <rPh sb="60" eb="62">
+      <t>ヒダリハジ</t>
+    </rPh>
+    <rPh sb="63" eb="65">
+      <t>トウタツ</t>
+    </rPh>
+    <rPh sb="70" eb="71">
+      <t>ダン</t>
+    </rPh>
+    <rPh sb="75" eb="77">
+      <t>ゲンザイ</t>
+    </rPh>
+    <rPh sb="78" eb="79">
+      <t>ダン</t>
+    </rPh>
+    <rPh sb="82" eb="84">
+      <t>ジョウダン</t>
+    </rPh>
+    <rPh sb="84" eb="87">
+      <t>サイコウビ</t>
+    </rPh>
+    <rPh sb="91" eb="93">
+      <t>イドウ</t>
+    </rPh>
+    <rPh sb="94" eb="96">
+      <t>ゲダン</t>
+    </rPh>
+    <rPh sb="96" eb="98">
+      <t>サイゼン</t>
+    </rPh>
+    <rPh sb="102" eb="104">
+      <t>イドウ</t>
+    </rPh>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>Fixedブクマの作成先は「ブックマーク」パネルでCtrl押しながらLclickで選択したブクマ・フォルダーにする。通常のLclickで選択しても、Fixedブクマの作成先の変更はしない。</t>
+    <rPh sb="9" eb="11">
+      <t>サクセイ</t>
+    </rPh>
+    <rPh sb="11" eb="12">
+      <t>サキ</t>
+    </rPh>
+    <rPh sb="29" eb="30">
+      <t>オ</t>
+    </rPh>
+    <rPh sb="41" eb="43">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="58" eb="60">
+      <t>ツウジョウ</t>
+    </rPh>
+    <rPh sb="68" eb="70">
+      <t>センタク</t>
+    </rPh>
+    <rPh sb="83" eb="85">
+      <t>サクセイ</t>
+    </rPh>
+    <rPh sb="85" eb="86">
+      <t>サキ</t>
+    </rPh>
+    <rPh sb="87" eb="89">
+      <t>ヘンコウ</t>
+    </rPh>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>メディアのページ数違いによる1ページの重みが♥1つに対応していないので、せめて、「同人誌、雑誌・アンソロジー、PRパンフ、切り取り本」の4分類ぐらいでFixedブクマの数を数えて♥の数を決めることとする。</t>
+    <rPh sb="8" eb="9">
+      <t>スウ</t>
+    </rPh>
+    <rPh sb="9" eb="10">
+      <t>チガ</t>
+    </rPh>
+    <rPh sb="19" eb="20">
+      <t>オモ</t>
+    </rPh>
+    <rPh sb="26" eb="28">
+      <t>タイオウ</t>
+    </rPh>
+    <rPh sb="41" eb="44">
+      <t>ドウジンシ</t>
+    </rPh>
+    <rPh sb="45" eb="47">
+      <t>ザッシ</t>
+    </rPh>
+    <rPh sb="61" eb="62">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="63" eb="64">
+      <t>ト</t>
+    </rPh>
+    <rPh sb="65" eb="66">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="69" eb="71">
+      <t>ブンルイ</t>
+    </rPh>
+    <rPh sb="84" eb="85">
+      <t>カズ</t>
+    </rPh>
+    <rPh sb="86" eb="87">
+      <t>カゾ</t>
+    </rPh>
+    <rPh sb="91" eb="92">
+      <t>カズ</t>
+    </rPh>
+    <rPh sb="93" eb="94">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="10"/>
+  </si>
+  <si>
+    <t>1</t>
+    <phoneticPr fontId="10"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Yu Gothic"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="源ノ角ゴシック JP"/>
+      <family val="2"/>
+      <charset val="128"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1222,7 +1406,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1232,12 +1416,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE7FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1253,133 +1431,139 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1668,10 +1852,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999"/>
   <cols>
-    <col min="1" max="2" width="3.921875" style="29" customWidth="1"/>
+    <col min="1" max="2" width="3.921875" style="28" customWidth="1"/>
     <col min="3" max="3" width="4.69140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="56.84375" style="3" customWidth="1"/>
     <col min="5" max="5" width="5.3828125" style="4" bestFit="1" customWidth="1"/>
@@ -1704,10 +1888,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="50.6">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="32" t="s">
         <v>25</v>
       </c>
       <c r="C2" s="9" t="s">
@@ -1718,7 +1902,7 @@
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C3" s="9" t="s">
@@ -1726,7 +1910,7 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="32" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="9" t="s">
@@ -1734,7 +1918,7 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="32" t="s">
         <v>28</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1742,7 +1926,7 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="32" t="s">
         <v>29</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1750,7 +1934,7 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -1758,7 +1942,7 @@
       </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="32" t="s">
         <v>31</v>
       </c>
       <c r="C8" s="9" t="s">
@@ -1766,7 +1950,7 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="32" t="s">
         <v>32</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -1774,7 +1958,7 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="32" t="s">
         <v>33</v>
       </c>
       <c r="C10" s="9" t="s">
@@ -1782,10 +1966,10 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="29" t="s">
+      <c r="A11" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C11" s="9" t="s">
@@ -1793,10 +1977,10 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="67.45">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -1808,18 +1992,18 @@
       <c r="E12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="39" t="s">
+      <c r="F12" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="G12" s="38" t="s">
+      <c r="G12" s="37" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="33.75">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C13" s="9" t="s">
@@ -1836,10 +2020,10 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="101.2">
-      <c r="A14" s="29" t="s">
+      <c r="A14" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C14" s="9" t="s">
@@ -1856,10 +2040,10 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="50.6">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -1877,10 +2061,10 @@
       <c r="I15" s="16"/>
     </row>
     <row r="16" spans="1:10" ht="101.2">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C16" s="9" t="s">
@@ -1895,10 +2079,10 @@
       <c r="I16" s="3"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="31" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -1912,7 +2096,7 @@
       </c>
     </row>
     <row r="18" spans="1:10">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="31" t="s">
         <v>1</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -1923,10 +2107,10 @@
       </c>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C19" s="9" t="s">
@@ -1937,10 +2121,10 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="50.6">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -1955,10 +2139,10 @@
       <c r="H20" s="27"/>
     </row>
     <row r="21" spans="1:10" ht="50.6">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B21" s="33" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1975,7 +2159,7 @@
       </c>
     </row>
     <row r="22" spans="1:10" ht="118.05">
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="33" t="s">
         <v>1</v>
       </c>
       <c r="C22" s="9" t="s">
@@ -1984,8 +2168,8 @@
       <c r="D22" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="28">
-        <v>0.6</v>
+      <c r="E22" s="8" t="s">
+        <v>18</v>
       </c>
       <c r="F22" s="24" t="s">
         <v>69</v>
@@ -1997,406 +2181,467 @@
         <v>74</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="33.75">
-      <c r="A23" s="29" t="s">
+    <row r="23" spans="1:10" ht="50.6">
+      <c r="B23" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="20"/>
+    </row>
+    <row r="24" spans="1:10" ht="33.75">
+      <c r="A24" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="B24" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="7" t="s">
+      <c r="C24" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="134.9">
-      <c r="A24" s="9" t="s">
+    <row r="25" spans="1:10" ht="134.9">
+      <c r="A25" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="B25" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="C25" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E25" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G25" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="33.75">
-      <c r="A25" s="9" t="s">
+    <row r="26" spans="1:10" ht="33.75">
+      <c r="A26" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="34" t="s">
+      <c r="B26" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="C26" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="134.9">
-      <c r="A26" s="9" t="s">
+    <row r="27" spans="1:10" ht="134.9">
+      <c r="A27" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="34" t="s">
+      <c r="B27" s="33" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="24" t="s">
+      <c r="C27" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="24" t="s">
         <v>47</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="H26" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="J26" s="24" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="33.75">
-      <c r="A27" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B27" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F27" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="118.05">
+      <c r="F27" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="H27" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="J27" s="24" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="33.75">
       <c r="A28" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="33" t="s">
         <v>66</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="24" t="s">
-        <v>56</v>
+      <c r="F28" s="15" t="s">
+        <v>57</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="I28" s="16" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="50.6">
-      <c r="A29" s="30" t="s">
-        <v>61</v>
-      </c>
-      <c r="B29" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="J28" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="118.05">
+      <c r="A29" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="33" t="s">
         <v>66</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D29" s="24" t="s">
-        <v>102</v>
+      <c r="D29" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F29" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="G29" s="36" t="s">
-        <v>97</v>
-      </c>
-      <c r="H29" s="35" t="s">
-        <v>95</v>
-      </c>
-      <c r="J29" s="20" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="67.45">
-      <c r="A30" s="31" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="I29" s="16" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="50.6">
+      <c r="A30" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="33" t="s">
         <v>66</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D30" s="21" t="s">
-        <v>64</v>
+      <c r="D30" s="24" t="s">
+        <v>102</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F30" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="J30" s="22" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="118.05">
-      <c r="A31" s="32" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="34" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="101.2">
-      <c r="A32" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="32" t="s">
-        <v>77</v>
+        <v>96</v>
+      </c>
+      <c r="G30" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="J30" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="50.6">
+      <c r="A31" s="29"/>
+      <c r="B31" s="44" t="s">
+        <v>130</v>
+      </c>
+      <c r="C31" s="9"/>
+      <c r="D31" s="42" t="s">
+        <v>129</v>
+      </c>
+      <c r="E31" s="43"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="34"/>
+      <c r="J31" s="20"/>
+    </row>
+    <row r="32" spans="1:10" ht="67.45">
+      <c r="A32" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>66</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="24" t="s">
-        <v>80</v>
+      <c r="D32" s="21" t="s">
+        <v>64</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F32" s="24" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>83</v>
+        <v>68</v>
+      </c>
+      <c r="J32" s="22" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="118.05">
-      <c r="A33" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="B33" s="32" t="s">
-        <v>77</v>
+      <c r="A33" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B33" s="33" t="s">
+        <v>0</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D33" s="24" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F33" s="24" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="50.6">
-      <c r="A34" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="B34" s="32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="101.2">
+      <c r="A34" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="31" t="s">
         <v>77</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>40</v>
       </c>
       <c r="D34" s="24" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E34" s="8" t="s">
         <v>18</v>
       </c>
       <c r="F34" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="G34" s="23" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="118.05">
+      <c r="A35" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="G35" s="23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="50.6">
+      <c r="A36" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B36" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="G34" s="23" t="s">
+      <c r="G36" s="23" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="50.6">
-      <c r="A35" s="32" t="s">
+    <row r="37" spans="1:8" ht="50.6">
+      <c r="A37" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="B35" s="32" t="s">
+      <c r="B37" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" s="24" t="s">
+      <c r="C37" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="24" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="32" t="s">
+    <row r="38" spans="1:8">
+      <c r="A38" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="D36" s="24" t="s">
+      <c r="D38" s="24" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="32" t="s">
+    <row r="39" spans="1:8">
+      <c r="A39" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="B37" s="32" t="s">
+      <c r="B39" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="39" t="s">
+      <c r="C39" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D39" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="H37" s="41" t="s">
+      <c r="E39" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H39" s="40" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="33.75">
-      <c r="A38" s="1"/>
-      <c r="B38" s="40" t="s">
+    <row r="40" spans="1:8" ht="33.75">
+      <c r="A40" s="1"/>
+      <c r="B40" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="C38" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D38" s="42" t="s">
+      <c r="C40" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D40" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="H38" s="37" t="s">
+      <c r="E40" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H40" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="1"/>
-      <c r="B39" s="40" t="s">
+    <row r="41" spans="1:8">
+      <c r="A41" s="1"/>
+      <c r="B41" s="39" t="s">
         <v>117</v>
       </c>
-      <c r="C39" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="42" t="s">
+      <c r="C41" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D41" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="H39" s="37" t="s">
+      <c r="E41" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H41" s="36" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="1"/>
-      <c r="B40" s="40" t="s">
-        <v>117</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D40" s="42" t="s">
+    <row r="42" spans="1:8" ht="269.8">
+      <c r="A42" s="1"/>
+      <c r="B42" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D42" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="H40" s="37"/>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="32" t="s">
+      <c r="E42" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F42" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="H42" s="36" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="31" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="32" t="s">
+      <c r="B43" s="39" t="s">
+        <v>126</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D43" s="38" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="50.6">
+      <c r="A44" s="31" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="32" t="s">
+      <c r="D44" s="42" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="31" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="32" t="s">
+    <row r="46" spans="1:8">
+      <c r="A46" s="31" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="32" t="s">
+    <row r="47" spans="1:8">
+      <c r="A47" s="31" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="32" t="s">
+    <row r="48" spans="1:8">
+      <c r="A48" s="31" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="32" t="s">
+    <row r="49" spans="1:1">
+      <c r="A49" s="31" t="s">
         <v>111</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="9"/>
+  <phoneticPr fontId="10"/>
   <hyperlinks>
-    <hyperlink ref="J29" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
+    <hyperlink ref="J30" r:id="rId1" location="12-1" xr:uid="{D7C16F2C-321A-4D1E-B495-101D7950FB2C}"/>
     <hyperlink ref="J22" r:id="rId2" location="64" xr:uid="{52043B27-C4EC-4B5C-9326-B5A0D68D6A6B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>